<commit_message>
Daily order sync: 2026-08-12
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M255"/>
+  <dimension ref="A1:M265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -859,17 +859,19 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 16:52:10 -0500</t>
+          <t>Tue, 11 Aug 2026 10:56:59 -0500</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 16:52:10 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19fafdd1abdd25b5]</t>
+          <t>Wed, 29 Jul 2026 16:52:10 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19fafdd1abdd25b5]
+Tue, 11 Aug 2026 10:56:59 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19ff18a97664b62d]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Hi, I did a very rough estimate and the price just for the regular front lit channel letter. However, there are many other details in installing, and specific materials about the sign that we will need</t>
+          <t>Hi, I did a very rough estimate and the price just for the regular front lit channel letter. However, there are many other details in installing, and specific materials about the sign that we will need
+Yes, working on it now! We will get back to you very soon. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile</t>
         </is>
       </c>
     </row>
@@ -928,7 +930,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -9930,15 +9932,20 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Wed, 22 Jul 2026 16:58:04 -0500</t>
+          <t>Tue, 11 Aug 2026 16:02:40 -0500</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>Wed, 22 Jul 2026 16:58:04 -0500: COI [19f8bd61c50f8a23]</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr"/>
+          <t>Wed, 22 Jul 2026 16:58:04 -0500: COI [19f8bd61c50f8a23]
+Tue, 11 Aug 2026 16:02:40 -0500: Re: Policies [19ff2a2943c206d5]</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Hi Michelle, We mailed the bond to the Board of Commissioners of Lake County 3 weeks ago, but have heard anything back yet. We have called the department but couldn&amp;#39;t connect to them. Do you know</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -9981,7 +9988,6 @@
           <t>Wed, 22 Jul 2026 16:57:31 -0500: Bond [19f8bd59cb6383fc]</t>
         </is>
       </c>
-      <c r="M203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -10447,7 +10453,6 @@
           <t>Wed, 22 Jul 2026 12:43:07 -0500: COI [19f8aecac6016c05]</t>
         </is>
       </c>
-      <c r="M213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -10490,7 +10495,6 @@
           <t>Wed, 22 Jul 2026 12:42:21 -0500: Bond [19f8aebf62f9288a]</t>
         </is>
       </c>
-      <c r="M214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -12416,6 +12420,476 @@
       <c r="M255" t="inlineStr">
         <is>
           <t>Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60632 www</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-0255</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Payment Awaiting</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>451 N Vine St - Permit Invoice</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>kchianelli@newlenox.net</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:59:28 +0000</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:59:28 +0000: 451 N Vine St - Permit Invoice [19ff2d6908d9737a]</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>Hello, The permit for the above property has been processed and is awaiting payment. Invoice number 00131403 can be paid online using our portal www.newlenox.net or in person Monday – Friday 8:30-5:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-0256</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Withdraw</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Confirmation of direct debit authorization for Village of Lisle</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>support@stripe.com</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:54:03 +0000</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:54:03 +0000: Confirmation of direct debit authorization for Village of Lisle [19ff2d1800803302]</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>Confirmation of direct debit authorization for Village of Lisle ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-0257</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Card Vault face lit trimless channel letters-Indy Re: Card Vault face lit trimless channel letters-Indy</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>mike@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:27:37 -0500 (CDT)</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:27:37 -0500 (CDT): Re: Card Vault face lit trimless channel letters-Indy [19ff2b94d1e89ad6]</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>There are 2 sets. One for each side of the building. $6400 for both? -----Original Message----- From: &amp;quot;charles zhao&amp;quot; &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Tuesday, August 11, 2026 3:06pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-0258</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Fw: Ziegler Re: Fw: Ziegler Re: Fw: Ziegler</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>zack.carpentersville@signarama.com</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:49:27 +0000</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:49:27 +0000: Re: Fw: Ziegler [19ff29678b58cd62]</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>See attached, it&amp;#39;s close to my home, let me now if you need better photos or video. I can stop by tomorrow morning. Zack Hermis Owner Office: 847-783-4870 Cell: 312-768-3529 Email: zack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-0259</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Still bending, Qi?</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>richard@omnimachineinc.com</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:47:25 -0700</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:47:25 -0700: Still bending, Qi? [19ff294a8c83d309]</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>Hi Qi, Been a few years since we quoted you on that GMC heavy-duty hydraulic box &amp;amp; pan brake — the 14 ga. x 120&amp;quot; machine. Wanted to check back in and see how the shop&amp;#39;s running. You got</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-0260</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Question about Workers Compensation Clearance Certificate  Application</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>osaemploymentcheck@dor.in.gov</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:08:22 -0500</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:08:22 -0500: Question about Workers Compensation Clearance Certificate  Application [19ff239c59ba0f68]</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Hi, Dear Indiana Department of Revenue I received a letter regarding missing documentation for my Workers&amp;#39; Compensation Clearance Certificate application. The letter states that I am missing an</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-0261</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Only) DH noodles&amp;grill PDF</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>topchannellettersorders@gmail.com</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:58:27 -0500</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:58:27 -0500: Re: (Estimate Only) DH noodles&amp;grill PDF [19ff1f9bcbeefbec]</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>On Tue, Aug 4, 2026 at 2:57 PM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-0262</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Sign Permit Application for Bedford Nail Spa, 7446 S. CICERO AVE BEDFORD PARK,IL 60629</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>ahuff@villageofbedfordpark.com</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:06:21 -0500</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:06:21 -0500: Re: Sign Permit Application for Bedford Nail Spa, 7446 S. CICERO AVE BEDFORD PARK,IL 60629 [19ff19320a13e772]</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>Hi Alyssa, Please let us know if you need anything else from us, Thank you so much for your help! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-0263</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Sign Proposal and Installation Agreement Re: Sign Proposal and Installation Agreement</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>dhurley580@aol.com</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:00:44 -0500</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:00:44 -0500: Re: Sign Proposal and Installation Agreement [19ff18dfa5602416]</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Thank you so much for your help! will process this sign. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile:</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-0264</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>[EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173 Re: [EXT] Re: Landlo</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>samantha.felling@simon.com</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:09:45 +0000</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:09:45 +0000: Re: [EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173 [19ff15f6777f909a]</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Hi Charles, I don&amp;#39;t see anything attached. Can you please resend it and cc simontctenantplans@simon.com? Thank you! Sammy Felling Tenant Coordinator Tenant Coordination The Simon® logo consisting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-13
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M265"/>
+  <dimension ref="A1:M283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1002,17 +1002,19 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 11:02:50 -0400</t>
+          <t>Wed, 12 Aug 2026 11:02:25 -0400</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 11:02:50 -0400: Renew Your Bond for Top Channel Letters Inc. [19ff15904d7036d2]</t>
+          <t>Tue, 11 Aug 2026 11:02:50 -0400: Renew Your Bond for Top Channel Letters Inc. [19ff15904d7036d2]
+Wed, 12 Aug 2026 11:02:25 -0400: Renew Your Bond for Top Channel Letters Inc. [19ff67f01ed139df]</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Dear qi zhao, Your $20000 IL License/Permit bond (#BX0073335) for Top Channel Letters Inc. is due for renewal on 09/11/2026. Your renewal has been approved at the following rate: Bond Term Cost Due Now</t>
+          <t>Dear qi zhao, Your $20000 IL License/Permit bond (#BX0073335) for Top Channel Letters Inc. is due for renewal on 09/11/2026. Your renewal has been approved at the following rate: Bond Term Cost Due Now
+Dear qi zhao, Your $10000 IL License/Permit bond (#BX0072566) for Top Channel Letters Inc. is due for renewal on 08/26/2026. Your renewal has been approved at the following rate: Bond Term Cost Due Now</t>
         </is>
       </c>
     </row>
@@ -12691,17 +12693,19 @@
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 14:08:22 -0500</t>
+          <t>Wed, 12 Aug 2026 14:19:50 +0000</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 14:08:22 -0500: Question about Workers Compensation Clearance Certificate  Application [19ff239c59ba0f68]</t>
+          <t>Tue, 11 Aug 2026 14:08:22 -0500: Question about Workers Compensation Clearance Certificate  Application [19ff239c59ba0f68]
+Wed, 12 Aug 2026 14:19:50 +0000: Re: Question about Workers Compensation Clearance Certificate Application [19ff6580fb63e147]</t>
         </is>
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>Hi, Dear Indiana Department of Revenue I received a letter regarding missing documentation for my Workers&amp;#39; Compensation Clearance Certificate application. The letter states that I am missing an</t>
+          <t>Hi, Dear Indiana Department of Revenue I received a letter regarding missing documentation for my Workers&amp;#39; Compensation Clearance Certificate application. The letter states that I am missing an
+Hello, Please submit your state tax filings. JENNIFER ERVIN TAX ANALYST 4 / TITLES AND CLEARANCES INDIANA DEPARTMENT OF REVENUE INDIANAPOLIS, IN 46241 FAX: 317-615-2736 From: charles zhao &amp;lt;</t>
         </is>
       </c>
     </row>
@@ -12890,6 +12894,852 @@
       <c r="M265" t="inlineStr">
         <is>
           <t>Hi Charles, I don&amp;#39;t see anything attached. Can you please resend it and cc simontctenantplans@simon.com? Thank you! Sammy Felling Tenant Coordinator Tenant Coordination The Simon® logo consisting</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-0265</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Only) H2O Interior Sign</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:56:22 -0700</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:56:22 -0700: (Estimate Only) H2O Interior Sign [19ff8311a2950158]</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>内部发光字 65.35&amp;#39;&amp;#39;x20&amp;#39;&amp;#39; 客人要和之前the one一样的材质 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-0266</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Only) Apex Spa Sign Re: (Estimate Only) Apex Spa Sign Re: (Estimate Only) Apex Spa Sign</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:55:51 -0500</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:55:51 -0500: Re: (Estimate Only) Apex Spa Sign [19ff7c2910600617]</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609 www</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-0267</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Sushi Hill Sign Production File (J)</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:27:57 -0700</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:27:57 -0700: Sushi Hill Sign Production File (J) [19ff8173a1d23216]</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>143.25&amp;#39;&amp;#39;x20&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-0268</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>rob@mnsignassoc.com</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT)</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ff8088e344e873]</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>Logo contest and sign design entries due by 08/28/2026! Minnesota Sign Association (MSA) REGISTRATION OPEN! ﻿ GLSA FALL CONFERENCE Register to join your industry peers for the inaugural conference of</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-0269</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>[EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>samantha.felling@simon.com</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:37:58 -0500</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:37:58 -0500: Re: [EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173 [19ff7e91f2dfc361]</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Hi, What do you say about the sign approval? Please let us know if you have any questions! We hope it can pass but also willing to adjust anything needed. Best Regards, Charles Zhao Top Channel Letters</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-0270</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>ilario@managechicago.com</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:35:05 -0500</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:35:05 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19ff7e67e0e6c91e]</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>Hi, Did you receive our invoice yesterday? Here is the file if you haven&amp;#39;t. Please let me know if you have any questions or further requests! We&amp;#39;d love to help. Best Regards, Charles Zhao Top</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-0271</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>PROJECT 31-2026 ( MOTIRAM)</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>getyoursigns@gmail.com</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:27:40 -0500</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:27:40 -0500: Re: PROJECT 31-2026 ( MOTIRAM) [19ff7dfb192cf6fa]</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Hi， What do you think of the new price? We agree with 200. We wanna develop a long term friendship with sign shops! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-0272</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Tupelo plans - Quote please REVISED QUOTE WITH NEW LOGO. Tupelo Q st revisions</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>jlane@alphasigns.us</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:16:10 -0500</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:16:10 -0500: Re: Tupelo plans - Quote please REVISED QUOTE WITH NEW LOGO. Tupelo Q st revisions [19ff7d52be629a9c]</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Hi Jason, What do you think of the price? We can negociate if you have any thoughts. We are using your design files, it looks a little different in the files we sent because we were trying to calculate</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-0273</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Back lit sign - family dental</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>info@signarama-schaumburg.com</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:13:18 -0500</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 16:13:18 -0500: Re: Back lit sign - family dental [19ff7d2887ab044f]</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>Hi, How are you doing? It has been a while since we sent the quote. What do you think of it? Please let me know if there&amp;#39;s anything you&amp;#39;d like to negociate. Hope you are having a good week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-0274</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Fast Sign Sign Production File (Yeuh)</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>topchannellettersorders@gmail.com</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:23:48 -0500</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:23:48 -0500: Re: Fast Sign Sign Production File (Yeuh) [19ff7a53b5aba3a8]</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>安裝管 这个颜色 Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-0275</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>PROJECT 29-2026 ( WINGSNOB CRYSTAL LAKE)</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>getyoursigns@gmail.com</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:06:30 -0500</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:06:30 -0500: Re: PROJECT 29-2026 ( WINGSNOB CRYSTAL LAKE) [19ff795e55a38fa5]</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>﻿ Hi, Chad spoke to you about this order. It needs a raceway and the color is sw 6071 popular gray. Please let&amp;#39;s get this done asap. Thank you Shannon On Tue, Jul 28, 2026 at 11:20 AM Fbs Prints</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-0276</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>(Permit Quote Needed)  for Wuliangye Restaurant 174 N Michigan Ave ,chicago Re: (Permit Quote Needed) for Wuliangye Rest</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>proimagepromotionsinc@gmail.com</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:00:26 -0500</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:00:26 -0500: Re: (Permit Quote Needed) for Wuliangye Restaurant 174 N Michigan Ave ,chicago [19ff790068acc936]</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>Hi Joy, This building is located in a special sign district, which only allows the tenant 144 sq ft of signage. Based on the image, this looks to be about ~300 sq ft, so the City will not permit about</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-0277</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>sftx62@gmail.com</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 12:53:30 -0700</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 12:53:30 -0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ff7897e7413a2e]</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>Hello Pat, Thanks for the feedback. We updated the rendering based on your comments. For the “THAI TWIST” returns, we recommend changing the return finish to white, with a 3&amp;quot; return depth. The</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-0278</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>"FASTSIGNS" sign Re: RFQ - "FASTSIGNS" sign</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>fastsigns.447@fastsigns.com</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 13:32:23 -0500</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 13:32:23 -0500: Re: RFQ - "FASTSIGNS" sign [19ff73fbf1f11591]</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>Yes. This color will work. Ravi. On Wed, Aug 12, 2026 at 11:46 AM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi Ravi, Please see attached photo PMS 427 C and the color we have in the sign</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-0279</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>IMPORTANT INFORMATION</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>buildingpermits@naperville.il.us</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 13:36:14 -0400 (EDT)</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 13:36:14 -0400 (EDT): IMPORTANT INFORMATION [19ff70bf368a59a4]</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>You have a secure message, please view details below. CITY OF NAPERVILLE UPDATE BUILDING PERMIT CONTRACTORS UPDATE Address: 400 S. Eagle Street Naperville, IL 60540 https://www.naperville.il.us/</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-0280</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>JD Logistics US - Nationwide Warehouse Signage Inquiry JD Logistics US - Nationwide Warehouse Signage Inquiry RE: Re: JD</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>wenxiao.zhong.1@jd.com</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 17:33:38 +0000</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 17:33:38 +0000: RE: Re: JD Logistics US - Nationwide Warehouse Signage Inquiry [19ff709a646116c0]</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>赵总好， 很高兴与您通话。 附件中是我方要求的规格参数。 钟文骁 Wenxiao Zhong Procurement Specialist International Procurement Department, Central Procurement Center, CFO System, JD Group Mobile: +1 7867198893 E- mail: wenxiao.zhong</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-0281</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Sign permits for 451 Vine</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Pylon Sign</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>rgraefen@newlenox.net</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:53:27 +0000</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 15:53:27 +0000: Fw: Sign permits for 451 Vine [19ff6add92fc62f6]</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>This was sent to the applicant. Ray Graefen Chief Building Inspector (815) 462-6492 (office) (815) 462-6469 (fax) Village of New Lenox 1 Veterans Parkway New Lenox, Illinois 60451 www.newlenox.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-0282</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Sonic</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>rpederson@waukesha-wi.gov</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:55:17 -0400 (EDT)</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:55:17 -0400 (EDT): Sonic [19ff565ce06ee30d]</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>The latest news from the City of Waukesha Sonic the Hedgehog 3 This Monday, August 17 head to Cutler Park for a viewing of Sonic the Hedgehog 3! You&amp;#39;ll want to come early starting at 6pm for the</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-14
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M283"/>
+  <dimension ref="A1:M298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -859,19 +859,21 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 10:56:59 -0500</t>
+          <t>Thu, 13 Aug 2026 11:14:03 -0500</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>Wed, 29 Jul 2026 16:52:10 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19fafdd1abdd25b5]
-Tue, 11 Aug 2026 10:56:59 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19ff18a97664b62d]</t>
+Tue, 11 Aug 2026 10:56:59 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19ff18a97664b62d]
+Thu, 13 Aug 2026 11:14:03 -0500: Re: Quote Inquiry for 12–15 ft Non‑Illuminated Sign at 2450 W Hubbard [19ffbe6f524bb1cb]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
           <t>Hi, I did a very rough estimate and the price just for the regular front lit channel letter. However, there are many other details in installing, and specific materials about the sign that we will need
-Yes, working on it now! We will get back to you very soon. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile</t>
+Yes, working on it now! We will get back to you very soon. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile
+sure. let us know if you have any questions Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130</t>
         </is>
       </c>
     </row>
@@ -930,7 +932,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -955,17 +957,19 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 22:31:20 +0700</t>
+          <t>Thu, 13 Aug 2026 11:15:30 -0500</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 22:31:20 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ff1734a1184586]</t>
+          <t>Tue, 11 Aug 2026 22:31:20 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ff1734a1184586]
+Thu, 13 Aug 2026 11:15:30 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ffbe84b6b9d8a3]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Thank you, Charles! I really appreciate it. Please let me know once you&amp;#39;ve had a chance to check everything. Best Regards, Pat. On Tue, Aug 11, 2026 at 9:08 PM charles zhao &amp;lt;topchannelletters@</t>
+          <t>Thank you, Charles! I really appreciate it. Please let me know once you&amp;#39;ve had a chance to check everything. Best Regards, Pat. On Tue, Aug 11, 2026 at 9:08 PM charles zhao &amp;lt;topchannelletters@
+buddy we can do it for you for 4000 both the store front sign and pylon sign . for the page 6, no worry. That is just the standard form we use. to confirm with you , we will build it with white return</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2722,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Permit</t>
+          <t>Awaiting Estimate</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2743,17 +2747,19 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Thu, 6 Aug 2026 13:06:49 -0500</t>
+          <t>Thu, 13 Aug 2026 16:28:10 +0000</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Thu, 6 Aug 2026 13:06:49 -0500: COI and Bond Needed for Village of Bridgeview [19fd841a9269dfe5]</t>
+          <t>Thu, 6 Aug 2026 13:06:49 -0500: COI and Bond Needed for Village of Bridgeview [19fd841a9269dfe5]
+Thu, 13 Aug 2026 16:28:10 +0000: Re: COI and Bond Needed for Village of Bridgeview [19ffbf3f0c723335]</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Hi Alex We need COI and Bond for Village of Bridgeview 7500 SOUTH OKETO AVENUE • BRIDGEVIEW, ILLINOIS 60455 Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top</t>
+          <t>Hi Alex We need COI and Bond for Village of Bridgeview 7500 SOUTH OKETO AVENUE • BRIDGEVIEW, ILLINOIS 60455 Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top
+Alex Wan Karstens Financial 312-465-5963 https://karstensfinancial.com/about-us/ Want to set up a meeting? Click Here Want an immediate Auto, Home, Business, Health or Life quote? https://</t>
         </is>
       </c>
     </row>
@@ -3354,17 +3360,19 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Thu, 06 Aug 2026 02:18:09 -0400</t>
+          <t>Thu, 13 Aug 2026 02:22:58 -0400</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Thu, 06 Aug 2026 02:18:09 -0400: Monthly Bond Payment Receipt [19fd5b8e09e22081]</t>
+          <t>Thu, 06 Aug 2026 02:18:09 -0400: Monthly Bond Payment Receipt [19fd5b8e09e22081]
+Thu, 13 Aug 2026 02:22:58 -0400: Monthly Bond Payment Receipt [19ff9c9cbe17b4c2]</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Monthly Bond Payment Receipt Dear Top Channel Letters Inc.: We have received your monthly payment of $10 on 08-06-2026. Bond number AM0003041 for Top Channel Letters Inc. will remain active. Download</t>
+          <t>Monthly Bond Payment Receipt Dear Top Channel Letters Inc.: We have received your monthly payment of $10 on 08-06-2026. Bond number AM0003041 for Top Channel Letters Inc. will remain active. Download
+Monthly Bond Payment Receipt Dear Top Channel Letters Inc.: We have received your monthly payment of $10 on 08-13-2026. Bond number AX0002455 for Top Channel Letters Inc. will remain active. Download</t>
         </is>
       </c>
     </row>
@@ -9982,12 +9990,18 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Wed, 22 Jul 2026 16:57:31 -0500</t>
+          <t>Thu, 13 Aug 2026 17:04:56 -0500</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>Wed, 22 Jul 2026 16:57:31 -0500: Bond [19f8bd59cb6383fc]</t>
+          <t>Wed, 22 Jul 2026 16:57:31 -0500: Bond [19f8bd59cb6383fc]
+Thu, 13 Aug 2026 17:04:56 -0500: Re: Right of Way Bond/Surety Bond  needed for Village of La Grange, IL [19ffd28295f9fb54]</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609 www</t>
         </is>
       </c>
     </row>
@@ -13024,17 +13038,19 @@
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 15:27:57 -0700</t>
+          <t>Thu, 13 Aug 2026 11:27:39 -0500</t>
         </is>
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 15:27:57 -0700: Sushi Hill Sign Production File (J) [19ff8173a1d23216]</t>
+          <t>Wed, 12 Aug 2026 15:27:57 -0700: Sushi Hill Sign Production File (J) [19ff8173a1d23216]
+Thu, 13 Aug 2026 11:27:39 -0500: Re: Sushi Hill Sign Production File (J) [19ffbf367299326f]</t>
         </is>
       </c>
       <c r="M268" t="inlineStr">
         <is>
-          <t>143.25&amp;#39;&amp;#39;x20&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com</t>
+          <t>143.25&amp;#39;&amp;#39;x20&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com
+安装管附件的颜色！ Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL</t>
         </is>
       </c>
     </row>
@@ -13071,12 +13087,13 @@
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT)</t>
+          <t>Thu, 13 Aug 2026 15:12:21 -0400 (EDT)</t>
         </is>
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ff8088e344e873]</t>
+          <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ff8088e344e873]
+Thu, 13 Aug 2026 15:12:21 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ffc8a2a1707ef0]</t>
         </is>
       </c>
       <c r="M269" t="inlineStr">
@@ -13118,17 +13135,19 @@
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 16:37:58 -0500</t>
+          <t>Thu, 13 Aug 2026 17:08:46 -0500</t>
         </is>
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 16:37:58 -0500: Re: [EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173 [19ff7e91f2dfc361]</t>
+          <t>Wed, 12 Aug 2026 16:37:58 -0500: Re: [EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173 [19ff7e91f2dfc361]
+Thu, 13 Aug 2026 17:08:46 -0500: Re: [EXT] Re: Landlord Approval Needed for Digiso, Space F113A , 5 Woodfield Mall, Schaumburg, IL 60173 [19ffd2bb5a2294c6]</t>
         </is>
       </c>
       <c r="M270" t="inlineStr">
         <is>
-          <t>Hi, What do you say about the sign approval? Please let us know if you have any questions! We hope it can pass but also willing to adjust anything needed. Best Regards, Charles Zhao Top Channel Letters</t>
+          <t>Hi, What do you say about the sign approval? Please let us know if you have any questions! We hope it can pass but also willing to adjust anything needed. Best Regards, Charles Zhao Top Channel Letters
+Dear Samantha, We just want to follow up with digiso sign approval from landlord,can you please let us know if you have any questions Thanks a lot! Best Regards, Charles Zhao Top Channel Letters Top</t>
         </is>
       </c>
     </row>
@@ -13740,6 +13759,711 @@
       <c r="M283" t="inlineStr">
         <is>
           <t>The latest news from the City of Waukesha Sonic the Hedgehog 3 This Monday, August 17 head to Cutler Park for a viewing of Sonic the Hedgehog 3! You&amp;#39;ll want to come early starting at 6pm for the</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-0283</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Enlarging existing channel letters Fw: Enlarging existing channel letters Re: Fw: Enlarging existing channel letters</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>carpentersvilleil@signarama.com</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 16:56:10 -0500</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 16:56:10 -0500: Re: Fw: Enlarging existing channel letters [19ffd202ab0b9170]</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>I just check the file again. yes, the best price we can do is $2200 the letters font is not easy to make. take much longer time than regular font. let us know if you want us to process this order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-0284</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Only) Huang &amp; Hu 清水正东律师事务所 Sign</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:46:20 -0700</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:46:20 -0700: (Estimate Only) Huang &amp; Hu 清水正东律师事务所 Sign [19ffd175ffbd12c6]</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-0285</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Angry Gene's Pizza Removal/Install Re: Angry Gene's Pizza Removal/Install Re: Angry Gene's Pizza Removal/Install Angry G</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>carpentersvilleil@signarama.com</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 19:36:53 +0000</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 19:36:53 +0000: Re: Angry Gene's Pizza Removal/Install [19ffca0b4f59c8f9]</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Perfect, we can keep the brackets just need raceway and channel letters. Just wanted to point that out. Signarama Team Office: 847-783-4870 Email: CarpentersvilleIL@signarama.com 58 E Main Street</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-0286</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Automatic reply: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Canopy</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>vaughn</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 21:34:37 +0000</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 21:34:37 +0000: Automatic reply: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [19ffd0c7d7163acb]</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Greetings! Please note that I am out of the office for the remainder of the day, Thursday, August 13, returning Monday, August 17. If you need immediate assistance in my absence, please contact Julie</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-0287</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>vaughn</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 16:34:20 -0500</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 16:34:20 -0500: Re: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [19ffd0c26e0fffd5]</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Hi, Jessica Sorry for late response Would you and Chrissy still available on Tuesday, August 18 at 11 AM, 1:30 PM, 2:30 PM Thank you for assistance Best Regards, Charles Zhao Top Channel Letters Top</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-0288</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Only) Angry Gene's Pizza Sign</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:13:50 -0700</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:13:50 -0700: (Estimate Only) Angry Gene's Pizza Sign [19ffcf99a6e310b2]</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-0289</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Chubby Cattle Woodfield Mall Temporary Banner Re: [EXT] Chubby Cattle Woodfield Mall Temporary Banner Re: [EXT] Chubby C</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Wayfinding</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>cspeca@simon.com</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 19:09:15 +0000</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 19:09:15 +0000: Re: [EXT] Chubby Cattle Woodfield Mall Temporary Banner [19ffc876546343ed]</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>We do not permit banners to be installed, and the property&amp;#39;s REA with Department stores do not permit us to do so. Christopher J. Speca General Manager Woodfield Mall 5 Woodfield Mall Schaumburg,</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-0290</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Payment Awaiting</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Wensco Sign Supply - Invoice# 4023902</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>ar@wensco.com</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 15:08:15 -0400</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 15:08:15 -0400: Wensco Sign Supply - Invoice# 4023902 [19ffc868e011a9d2]</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Billing Contact TOP CHANNEL LETTERS INC See attached file(s). Kay James Wensco Sign Supply ar@wensco.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-0291</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Payment Awaiting</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Wensco Sign Supply - Invoice# 4023900</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>ar@wensco.com</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 15:06:56 -0400</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 15:06:56 -0400: Wensco Sign Supply - Invoice# 4023900 [19ffc8561054d0e4]</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Billing Contact TOP CHANNEL LETTERS INC See attached file(s). Kay James Wensco Sign Supply ar@wensco.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-0292</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Re: JD Logistics US - Nationwide Warehouse Signage Inquiry Re: Re: Re: JD Logistics US - Nationwide Warehouse Signage In</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>wenxiao.zhong.1@jd.com</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 16:37:25 +0000</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 16:37:25 +0000: RE: Re: Re: JD Logistics US - Nationwide Warehouse Signage Inquiry [19ffbfc89cacef20]</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>赵总， 效果图请见附件。 这个材料是总部确认过的，我理解厚度填充是厚泡沫板即可。 钟文骁 Wenxiao Zhong Procurement Specialist International Procurement Department, Central Procurement Center, CFO System, JD Group Mobile: +1 7867198893 E- mail:</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-0293</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>General Email</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>manfredis@lyndhurstohio.gov</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 09:26:53 -0700 (MST)</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 09:26:53 -0700 (MST): General Email [19ffbf2ae2b7d744]</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Your permit is ready for payment. Please go to the portal and make payment. Portal: CLICK HERE Best, Sheila Manfredi Administrative Assistant 440-473-5108 manfredis@lyndhurstohio.gov</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-0294</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Payment received: Invoice #182686-(Chi Tung)</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>quickbooks@notification.intuit.com</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:55:13 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:55:13 +0000 (UTC): Payment received: Invoice #182686-(Chi Tung) [19ffb9ec7df43f33]</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Intuit QuickBooks View sale $3575.38 Payment has been received Payment details Paid to Top Channel Letters Customer name Chi Tung Customer email Firstchicago209@gmail.com Invoice no. 182686 Paid date</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-0295</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Clark County Nevada Accela Update</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>ADA Signage</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>clark county</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:33:08 +0000</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 14:33:08 +0000: Clark County Nevada Accela Update [19ffb8a8bb0e643f]</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Dear Valued Customer, This email is to inform you of a scheduled Clark County-wide network maintenance outage that will occur beginning Friday, August 28, 2026, at 11:00 PM through Saturday, August 29,</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-0296</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Your free trial ends tomorrow</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>email@email.shopify.com</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 06:00:29 +0000</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 06:00:29 +0000: Your free trial ends tomorrow [19ff9b5337f51c3f]</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Sign up to earn 1% back on all sales ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-0297</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Signage Flex Spec Guide -- LED neon flex for Top Channel Letters</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>winston@etnlighting.com</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 13:39:53 +0800 (CST)</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Thu, 13 Aug 2026 13:39:53 +0800 (CST): Signage Flex Spec Guide -- LED neon flex for Top Channel Letters [19ff9a2748783ff0]</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Hi Top Channel Letters Team, I&amp;#39;ve been looking closely at Top Channel Letters&amp;#39;s illuminated channel letters and sign fabrication--particularly how your sign installations require bright,</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-17
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M306"/>
+  <dimension ref="A1:M322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -932,7 +932,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Payment Awaiting</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -957,19 +957,21 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Thu, 13 Aug 2026 11:15:30 -0500</t>
+          <t>Sun, 16 Aug 2026 22:28:29 -0500</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>Tue, 11 Aug 2026 22:31:20 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ff1734a1184586]
-Thu, 13 Aug 2026 11:15:30 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ffbe84b6b9d8a3]</t>
+Thu, 13 Aug 2026 11:15:30 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ffbe84b6b9d8a3]
+Sun, 16 Aug 2026 22:28:29 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a00dc37655eb712]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>Thank you, Charles! I really appreciate it. Please let me know once you&amp;#39;ve had a chance to check everything. Best Regards, Pat. On Tue, Aug 11, 2026 at 9:08 PM charles zhao &amp;lt;topchannelletters@
-buddy we can do it for you for 4000 both the store front sign and pylon sign . for the page 6, no worry. That is just the standard form we use. to confirm with you , we will build it with white return</t>
+buddy we can do it for you for 4000 both the store front sign and pylon sign . for the page 6, no worry. That is just the standard form we use. to confirm with you , we will build it with white return
+i think either white return with white trim cap will work fine . or black return with black trim cap will be good as well. it will give like an outline for the sign. for the raceway #8 is ok. our white</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1173,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1196,17 +1198,19 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Wed, 5 Aug 2026 14:20:15 -0400</t>
+          <t>Sun, 16 Aug 2026 22:42:26 -0500</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Wed, 5 Aug 2026 14:20:15 -0400: Re: TopChannelLetters - Referred by Jovim from inoprints [19fd327c4360bcd0]</t>
+          <t>Wed, 5 Aug 2026 14:20:15 -0400: Re: TopChannelLetters - Referred by Jovim from inoprints [19fd327c4360bcd0]
+Sun, 16 Aug 2026 22:42:26 -0500: Re: TopChannelLetters - Referred by Jovim from inoprints [1a00dd03bb458bb8]</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Can I send someone to measure the building size ? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404</t>
+          <t>Can I send someone to measure the building size ? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404
+HI, Yosf, Please check the sample of the backlit channel letters we made for other businesses. Do you like the silver color or the gold color? and do you think you can stop by our sign shop and talk</t>
         </is>
       </c>
     </row>
@@ -3127,17 +3131,19 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Wed, 5 Aug 2026 21:20:10 +0000</t>
+          <t>Mon, 17 Aug 2026 16:33:06 +0000</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Wed, 5 Aug 2026 21:20:10 +0000: RE: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [19fd3cc6629145c7]</t>
+          <t>Wed, 5 Aug 2026 21:20:10 +0000: RE: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [19fd3cc6629145c7]
+Mon, 17 Aug 2026 16:33:06 +0000: RE: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [1a01091e4efc54ba]</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Charles, Monday, August 10 would be best, Chrissy and I are both available at 3 PM. Let me know if that works and I can send a virtual meeting invite. Best, Jessica Jessica Vaughn, AICP (she/her) Urban</t>
+          <t>Charles, Monday, August 10 would be best, Chrissy and I are both available at 3 PM. Let me know if that works and I can send a virtual meeting invite. Best, Jessica Jessica Vaughn, AICP (she/her) Urban
+Charles, It does not look like I am available at that time any longer. How about Wednesday, at 10:30 AM? Jessica Vaughn, AICP (she/her) Urban Design Commission Secretary – Planning Division Department</t>
         </is>
       </c>
     </row>
@@ -5855,12 +5861,13 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 19:45:46 +0000 (UTC)</t>
+          <t>Sat, 15 Aug 2026 00:45:02 +0000 (UTC)</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 19:45:46 +0000 (UTC): Your Items have Shipped! [19fb48fbe3b3d879]</t>
+          <t>Thu, 30 Jul 2026 19:45:46 +0000 (UTC): Your Items have Shipped! [19fb48fbe3b3d879]
+Sat, 15 Aug 2026 00:45:02 +0000 (UTC): Your Items have Shipped! [1a002e121e032510]</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
@@ -6043,19 +6050,21 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 18:56:53 +0000</t>
+          <t>Sun, 16 Aug 2026 14:55:11 -0500</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
         <is>
           <t>Thu, 30 Jul 2026 18:16:54 +0000: Re: Possible Inquiry [19fb43e8077894c3]
-Fri, 14 Aug 2026 18:56:53 +0000: Re: Possible Inquiry [1a001a269f531fda]</t>
+Fri, 14 Aug 2026 18:56:53 +0000: Re: Possible Inquiry [1a001a269f531fda]
+Sun, 16 Aug 2026 14:55:11 -0500: Re: Possible Inquiry [1a00c247507b8dbd]</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
         <is>
           <t>This would be the final design. Signarama Team Office: 815-744-8702 Email: JolietIL@signarama.com 1107 Essington Road Joliet, IL 60435 www.signarama-joliet.com View our entire catalog here! Please
-The client will take care of the fees, just let me know the pricing for the fees and what not. You told me $1350. Signarama Team Office: 815-744-8702 Email: JolietIL@signarama.com 1107 Essington Road</t>
+The client will take care of the fees, just let me know the pricing for the fees and what not. You told me $1350. Signarama Team Office: 815-744-8702 Email: JolietIL@signarama.com 1107 Essington Road
+let us see installation is 850, remove old sign is 200 Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile:</t>
         </is>
       </c>
     </row>
@@ -11168,17 +11177,19 @@
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>Wed, 22 Jul 2026 00:02:58 -0400</t>
+          <t>Sun, 16 Aug 2026 00:04:22 -0400</t>
         </is>
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>Wed, 22 Jul 2026 00:02:58 -0400: [Follow Up] Bond Quote for Top Channel Letters Inc. [19f87fdbb4898a79]</t>
+          <t>Wed, 22 Jul 2026 00:02:58 -0400: [Follow Up] Bond Quote for Top Channel Letters Inc. [19f87fdbb4898a79]
+Sun, 16 Aug 2026 00:04:22 -0400: [Follow Up] Bond Quote for Top Channel Letters Inc [1a008bdfd140fef6]</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>We recently quoted a IL Contractor&amp;#39;s License/Permit bond for you. You are approved for the following bond quote and can proceed with the purchase by clicking the button below: Bond Term Cost</t>
+          <t>We recently quoted a IL Contractor&amp;#39;s License/Permit bond for you. You are approved for the following bond quote and can proceed with the purchase by clicking the button below: Bond Term Cost
+We recently quoted a IL License/Permit bond for you. You are approved for the following bond quote and can proceed with the purchase by clicking the button below: Bond Term Cost Due Now Monthly $10 $60</t>
         </is>
       </c>
     </row>
@@ -11926,13 +11937,15 @@
       <c r="L244" t="inlineStr">
         <is>
           <t>Tue, 21 Jul 2026 14:25:16 -0500: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [19f8623b9f970dab]
-Fri, 14 Aug 2026 16:19:24 -0500: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a00224d432e9243]</t>
+Fri, 14 Aug 2026 16:19:24 -0500: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a00224d432e9243]
+Mon, 17 Aug 2026 21:22:12 +0000: RE: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a0119a9d601f480]</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
           <t>Hi, Martin We are Top Channel Letters, the sign contractor for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 We would like to apply for a sign permit for this business. The attachments include
-Hi, Lisa This is the revision for sign 3, we have updated a smaller sign to fit the requirement. Please check. Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top</t>
+Hi, Lisa This is the revision for sign 3, we have updated a smaller sign to fit the requirement. Please check. Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top
+Good Afternoon, Please refer to the attached letter that our Chief Building Inspector, Ray Graefen sent regarding the review your signs. We are still in need of a response letter with electrical</t>
         </is>
       </c>
     </row>
@@ -12864,17 +12877,19 @@
       </c>
       <c r="K264" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 11:00:44 -0500</t>
+          <t>Sun, 16 Aug 2026 22:21:16 -0500</t>
         </is>
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>Tue, 11 Aug 2026 11:00:44 -0500: Re: Sign Proposal and Installation Agreement [19ff18dfa5602416]</t>
+          <t>Tue, 11 Aug 2026 11:00:44 -0500: Re: Sign Proposal and Installation Agreement [19ff18dfa5602416]
+Sun, 16 Aug 2026 22:21:16 -0500: Re: Sign Proposal and Installation Agreement [1a00dbcdabb711c5]</t>
         </is>
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>Thank you so much for your help! will process this sign. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile:</t>
+          <t>Thank you so much for your help! will process this sign. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile:
+Dear Donald, Thanks for your reply. we will talk to the business owner and start production Thanks! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:</t>
         </is>
       </c>
     </row>
@@ -13108,7 +13123,8 @@
         <is>
           <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ff8088e344e873]
 Thu, 13 Aug 2026 15:12:21 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ffc8a2a1707ef0]
-Fri, 14 Aug 2026 12:46:31 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a0012b032f8c76d]</t>
+Fri, 14 Aug 2026 12:46:31 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a0012b032f8c76d]
+Sat, 15 Aug 2026 10:57:47 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a005edd40ae423a]</t>
         </is>
       </c>
       <c r="M269" t="inlineStr">
@@ -13581,17 +13597,19 @@
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 13:32:23 -0500</t>
+          <t>Sun, 16 Aug 2026 18:53:31 -0500</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 13:32:23 -0500: Re: RFQ - "FASTSIGNS" sign [19ff73fbf1f11591]</t>
+          <t>Wed, 12 Aug 2026 13:32:23 -0500: Re: RFQ - "FASTSIGNS" sign [19ff73fbf1f11591]
+Sun, 16 Aug 2026 18:53:31 -0500: Re: RFQ - "FASTSIGNS" sign [1a00cfea99cd6084]</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Yes. This color will work. Ravi. On Wed, Aug 12, 2026 at 11:46 AM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi Ravi, Please see attached photo PMS 427 C and the color we have in the sign</t>
+          <t>Yes. This color will work. Ravi. On Wed, Aug 12, 2026 at 11:46 AM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi Ravi, Please see attached photo PMS 427 C and the color we have in the sign
+Finally we got the vinyl . There is still a problem with the supplier , they sent us a 48&amp;quot;x50yards roll .crazy.! I will have this job completed very soon. do not remember if you need us to install</t>
         </is>
       </c>
     </row>
@@ -14522,17 +14540,19 @@
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 17:01:14 -0500</t>
+          <t>Sun, 16 Aug 2026 23:02:52 -0500</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 17:01:14 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0024b5160293ad]</t>
+          <t>Fri, 14 Aug 2026 17:01:14 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0024b5160293ad]
+Sun, 16 Aug 2026 23:02:52 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a00de2eea056286]</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>Hello Charles, I am in the process of opening a new Stretch Zone studio at 1733 W. Kirby Avenue in Champaign and would like to request a proposal for the fabrication and installation of our exterior</t>
+          <t>Hello Charles, I am in the process of opening a new Stretch Zone studio at 1733 W. Kirby Avenue in Champaign and would like to request a proposal for the fabrication and installation of our exterior
+Hi, is this sport clip your shop? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W</t>
         </is>
       </c>
     </row>
@@ -14663,17 +14683,19 @@
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 17:21:06 +0000</t>
+          <t>Mon, 17 Aug 2026 13:45:22 +0000</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 17:21:06 +0000: Re: Enlarging existing channel letters [1a0014ac72caa072]</t>
+          <t>Fri, 14 Aug 2026 17:21:06 +0000: Re: Enlarging existing channel letters [1a0014ac72caa072]
+Mon, 17 Aug 2026 13:45:22 +0000: Re: Enlarging existing channel letters [1a00ff86385fac0b]</t>
         </is>
       </c>
       <c r="M302" t="inlineStr">
         <is>
-          <t>Charles. We would like to proceed. Get Outlook for iOS From: charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Thursday, 13 August 2026 16:56:10 To: Signarama Carptenersville IL &amp;lt;</t>
+          <t>Charles. We would like to proceed. Get Outlook for iOS From: charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Thursday, 13 August 2026 16:56:10 To: Signarama Carptenersville IL &amp;lt;
+Good morning, Charles See below and yes, I will prepare a check and send you a picture today. Also, around Noon-2oclock I will go by Zeigler&amp;#39;s and facetime you. See info below for Angry genes</t>
         </is>
       </c>
     </row>
@@ -14710,17 +14732,19 @@
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 12:47:14 -0500</t>
+          <t>Mon, 17 Aug 2026 12:28:53 +0000</t>
         </is>
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 12:47:14 -0500: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a00162959aa0e3e]</t>
+          <t>Fri, 14 Aug 2026 12:47:14 -0500: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a00162959aa0e3e]
+Mon, 17 Aug 2026 12:28:53 +0000: RE: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a00fb258a5a2c48]</t>
         </is>
       </c>
       <c r="M303" t="inlineStr">
         <is>
-          <t>Dear Town Hall, We are Top Channel Letters, the sign contractor for Nori Sushi &amp;amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 We would like to apply for a sign permit for this business. The</t>
+          <t>Dear Town Hall, We are Top Channel Letters, the sign contractor for Nori Sushi &amp;amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 We would like to apply for a sign permit for this business. The
+Hi Charles ~ Thank you for this information! I apologize, but the form you filled out for a sign request pertains to our sign out front, if residents want to put something on our sign (I can see the</t>
         </is>
       </c>
     </row>
@@ -14862,6 +14886,758 @@
       <c r="M306" t="inlineStr">
         <is>
           <t>Attached is a PDF containing your Sherwin-Williams Invoices. If you have any questions regarding your invoices, please contact our Financial Services team at 800-782-4660. This email (including any</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-0306</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Presotea - Sign Info Presotea - Sign Info Re: Presotea - Sign Info Re: Presotea - Sign Info Re: Presotea - Sign Info Re:</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>tony liu</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 21:44:25 -0500</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 21:44:25 -0500: Re: Presotea - Sign Info [1a00d9b1ff6718ae]</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>Hi Tony, can you give me a call to discuss? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-0307</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Com Electrical Permit PCE26-0087 with VILLAGE OF HILLSIDE Issued</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>adnandavid27@yahoo.com</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 17:43:18 -0500</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 17:43:18 -0500: Fwd: Com Electrical Permit PCE26-0087 with VILLAGE OF HILLSIDE Issued [1a011e54380a87a3]</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>Sent from my iPhone Begin forwarded message: From: VILLAGE OF HILLSIDE - Community Development &amp;lt;noreply@bsacloud.com&amp;gt; Date: August 17, 2026 at 3:02:33 PM CDT To: topchannelletters@gmail.com,</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-0308</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Sign Rendering of your tanent Reset Bodywork Spa, 3032 Hobson Rd, Woodridge, IL 60517</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>kathryn@capitalrep.com</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 15:12:51 -0500</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 15:12:51 -0500: Re: Sign Rendering of your tanent Reset Bodywork Spa, 3032 Hobson Rd, Woodridge, IL 60517 [1a0115af614cecfc]</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>Hi，Kathryn Our team went Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-0309</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Landlord Approval Needed for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 Re: Landlord Approval Needed f</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>dspeth@midamericagrp.com</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 20:01:20 +0000</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 20:01:20 +0000: RE: Landlord Approval Needed for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a0115082ef41916]</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>Charles, I am not the LL im am the property manager, so you need to update the form for the owner to sign. Ownership: Brighton Greens LLC Contact: Timothy Peach Title: Owner Address: 14097 Frederick</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-0310</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Interior illuminated sign Interior illuminated sign</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>signarama woodridge</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 19:26:34 +0000</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 19:26:34 +0000: Interior illuminated sign [1a01130b8f9cdfdc]</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>Hi Charles, Could you please provide a production quote for an interior illuminated sign? A few details: Interior sign Back-lit / halo-lit No installation required, production only Approximate size: 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-0311</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Village of Hillside - Review Result for PCE26-0087</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>adnandavid27@yahoo.com</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 12:30:18 -0500</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 12:30:18 -0500: Fwd: Village of Hillside - Review Result for PCE26-0087 [1a010c6779da9e49]</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>Sent from my iPhone Begin forwarded message: &amp;gt; From: VILLAGE OF HILLSIDE - Community Development &amp;gt; Date: August 17, 2026 at 12:17:07 PM CDT &amp;gt; To: adnandavid27@yahoo.com &amp;gt; Subject: Village</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-0312</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Payment Awaiting</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Village of Hillside - Invoice Due for 4600 ROOSEVELT RD</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>adnandavid27@yahoo.com</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 12:29:51 -0500</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 12:29:51 -0500: Fwd: Village of Hillside - Invoice Due for 4600 ROOSEVELT RD [1a010c60125438c9]</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>Sent from my iPhone Begin forwarded message: From: VILLAGE OF HILLSIDE - Community Development &amp;lt;noreply@bsacloud.com&amp;gt; Date: August 17, 2026 at 12:16:47 PM CDT To: adnandavid27@yahoo.com Subject:</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-0313</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>August 17 Meeting of the Village Board</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>admin@public.govdelivery.com</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 17:01:35 +0000</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 17:01:35 +0000: August 17 Meeting of the Village Board [1a010abe5622252a]</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>Having trouble viewing this email? View it as a Web page. | Bookmark and Share MEETING OF THE VILLAGE BOARD Village Hall Village Hall 14700 S. Ravinia Ave, Orland Park, IL 60462 Monday, August 17, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-0314</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Save Time on Estimating—We'll Handle It</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>klemroshy9@gmail.com</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 09:08:10 -0700</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 09:08:10 -0700: Re: Save Time on Estimating—We'll Handle It [1a0107b2b76599b8]</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>Hi, Sorry to bother you again, This is just a follow up email. Have you received my emails? We are a cost estimating service provider all over the USA. Our estimation team is working around the clock</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-0315</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Correspondence from Village of Downers Grove - Permit Review Corrections Notice (26-PSG-0039)</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>cityview_donotreply@downers.us</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>17 Aug 2026 09:52:45 -0400</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>17 Aug 2026 09:52:45 -0400: Correspondence from Village of Downers Grove - Permit Review Corrections Notice (26-PSG-0039) [1a00fff023d1568c]</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>Please see attached document. This email was sent from Downers Grove Production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-0316</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Want to see how AI can do the heavy lifting for your store?</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>email@email.shopify.com</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 09:45:51 +0000</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 09:45:51 +0000: Want to see how AI can do the heavy lifting for your store? [1a00f1cf8624698a]</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>Launch your store faster with the help of AI tools. ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-0317</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Re: Re: JD Logistics US - Nationwide Warehouse Signage Inquiry</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>wenxiao.zhong.1@jd.com</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 00:17:38 -0500</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 00:17:38 -0500: Re: Re: Re: JD Logistics US - Nationwide Warehouse Signage Inquiry [1a00e2760b502f24]</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>钟总， 我计算了一下， 方案一做成我们正常的铝皮字 3“ 厚度的话，制作的价格大概在$3850. 工艺是这样的： Standard Channel Letters Acrylic faces with trimcaps .040 aluminum returns 这个是制作价格不包括邮寄或者安装。安装是要根据实际情况才报的了的。主要是看安装的难度，难度取决于安装的高度，和安装的技巧。如果很高的地方，</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-0318</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Completed: You're copied on "Bedford Nail Spa Pylon Sign Rendering 26-6"</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Pylon Sign</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>adobesign@adobesign.com</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 08:02:30 -0700 (PDT)</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 08:02:30 -0700 (PDT): Completed: You're copied on "Bedford Nail Spa Pylon Sign Rendering 26-6" [1a00b188536a5c50]</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>Attached is the final agreement for your reference. QA PRINTS cc&amp;#39;d you on Bedford Nail Spa Pylon Sign Rendering 26-6 Open agreement Attached is the final agreement between: QA PRINTS Donald T.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-0319</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Step 1: open this. Step 2 is inside.</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>email@email.shopify.com</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 09:45:50 +0000</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 09:45:50 +0000: Step 1: open this. Step 2 is inside. [1a009f697089dab2]</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>Sign up for a plan to keep building your store without interruption. ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-0320</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Get an additional 3 months of Shopify for $1/mo</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>email@email.shopify.com</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Sat, 15 Aug 2026 06:01:14 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Sat, 15 Aug 2026 06:01:14 +0000 (UTC): Get an additional 3 months of Shopify for $1/mo [1a004029bb453dc0]</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>Plus, earn up to $10000 in credits ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-0321</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Shinto(Ohio) Sign Production File (J)</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Fri, 14 Aug 2026 16:12:58 -0700</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Fri, 14 Aug 2026 16:12:58 -0700: Shinto(Ohio) Sign Production File (J) [1a0028d301649bbc]</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>1. 圆形灯箱 55&amp;#39;&amp;#39; 2. SHINTO 80.5&amp;#39;&amp;#39;x26.5&amp;#39;&amp;#39; 3. JAPANESE STEAKHOUSE &amp;amp; SUSHI 228&amp;#39;&amp;#39;x13&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-18
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M322"/>
+  <dimension ref="A1:M340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -957,21 +957,23 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Sun, 16 Aug 2026 22:28:29 -0500</t>
+          <t>Tue, 18 Aug 2026 10:52:03 +0700</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>Tue, 11 Aug 2026 22:31:20 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ff1734a1184586]
 Thu, 13 Aug 2026 11:15:30 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ffbe84b6b9d8a3]
-Sun, 16 Aug 2026 22:28:29 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a00dc37655eb712]</t>
+Sun, 16 Aug 2026 22:28:29 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a00dc37655eb712]
+Tue, 18 Aug 2026 10:52:03 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a012ff9cfedabf7]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>Thank you, Charles! I really appreciate it. Please let me know once you&amp;#39;ve had a chance to check everything. Best Regards, Pat. On Tue, Aug 11, 2026 at 9:08 PM charles zhao &amp;lt;topchannelletters@
 buddy we can do it for you for 4000 both the store front sign and pylon sign . for the page 6, no worry. That is just the standard form we use. to confirm with you , we will build it with white return
-i think either white return with white trim cap will work fine . or black return with black trim cap will be good as well. it will give like an outline for the sign. for the raceway #8 is ok. our white</t>
+i think either white return with white trim cap will work fine . or black return with black trim cap will be good as well. it will give like an outline for the sign. for the raceway #8 is ok. our white
+Hi Charles, Thank you for the update. I noticed that the Zelle transfer option is not available on my account yet. I&amp;#39;m currently setting it up with the bank, which may take 1–2 business days. I</t>
         </is>
       </c>
     </row>
@@ -9626,17 +9628,19 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Thu, 23 Jul 2026 15:43:17 +0000</t>
+          <t>Tue, 18 Aug 2026 10:07:05 -0500</t>
         </is>
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>Thu, 23 Jul 2026 15:43:17 +0000: RE: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [19f8fa55306c33f2]</t>
+          <t>Thu, 23 Jul 2026 15:43:17 +0000: RE: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [19f8fa55306c33f2]
+Tue, 18 Aug 2026 10:07:05 -0500: Re: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a015695e8912f87]</t>
         </is>
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>Good Morning, Thank you for your submittal. I have processed the permits and they are currently awaiting review. We will contact you should we need anything further. Lisa Martin Senior Administrative</t>
+          <t>Good Morning, Thank you for your submittal. I have processed the permits and they are currently awaiting review. We will contact you should we need anything further. Lisa Martin Senior Administrative
+got it, thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9934,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Permit</t>
+          <t>Awaiting Estimate</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -9955,7 +9959,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 12:59:19 +0000</t>
+          <t>Tue, 18 Aug 2026 15:59:01 -0500</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -9964,7 +9968,10 @@
 Tue, 11 Aug 2026 16:02:40 -0500: Re: Policies [19ff2a2943c206d5]
 Fri, 14 Aug 2026 20:38:30 +0000: Re: Right of Way Bond/Surety Bond needed for Village of La Grange, IL [1a001ff7556c09b2]
 Fri, 14 Aug 2026 16:14:52 +0000: Chicago Open House - August 20th [1a0010e31b7e8f81]
-Fri, 14 Aug 2026 12:59:19 +0000: RE: Policies [1a0005b0c286f06f]</t>
+Fri, 14 Aug 2026 12:59:19 +0000: RE: Policies [1a0005b0c286f06f]
+Tue, 18 Aug 2026 16:29:20 -0500: Life Space Digital Invoice &amp; COI from Top Channel Letters [1a016c764718db5d]
+Tue, 18 Aug 2026 16:13:42 -0500: Fwd: coi [1a016b94677bc643]
+Tue, 18 Aug 2026 15:59:01 -0500: Fwd: coi [1a016abd350fc6d3]</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -9972,7 +9979,10 @@
           <t>Hi Michelle, We mailed the bond to the Board of Commissioners of Lake County 3 weeks ago, but have heard anything back yet. We have called the department but couldn&amp;#39;t connect to them. Do you know
 Alex Wan Karstens Financial 312-465-5963 https://karstensfinancial.com/about-us/ Want to set up a meeting? Click Here Want an immediate Auto, Home, Business, Health or Life quote? https://
 Hello, Just a quick reminder that Grimco&amp;#39;s Open House at our Chicago facility (Bolingbrook, IL) is coming up on Thursday, August 20th, and we&amp;#39;d love to see you there. This is a great
-Please call 219 755 3730. This is the number to our recorder&amp;#39;s office. They aren&amp;#39;t even located within the same town as me. They should be able to help you. From: charles zhao &amp;lt;</t>
+Please call 219 755 3730. This is the number to our recorder&amp;#39;s office. They aren&amp;#39;t even located within the same town as me. They should be able to help you. From: charles zhao &amp;lt;
+Dear Sunny, Please see attached invoice and COI. Feel free to contact us if you have any questions. Thank you! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:
+---------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 4:10 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan
+---------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 3:53 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan</t>
         </is>
       </c>
     </row>
@@ -9984,7 +9994,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Permit</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -10009,20 +10019,23 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 16:09:45 -0400</t>
+          <t>Tue, 18 Aug 2026 15:16:17 -0500</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
         <is>
           <t>Wed, 22 Jul 2026 16:57:31 -0500: Bond [19f8bd59cb6383fc]
 Thu, 13 Aug 2026 17:04:56 -0500: Re: Right of Way Bond/Surety Bond  needed for Village of La Grange, IL [19ffd28295f9fb54]
-Fri, 14 Aug 2026 16:09:45 -0400: Bond Quote for Top Channel Letters Inc [1a001e51ba1b2a17]</t>
+Fri, 14 Aug 2026 16:09:45 -0400: Bond Quote for Top Channel Letters Inc [1a001e51ba1b2a17]
+Tue, 18 Aug 2026 16:36:45 -0400: Bond Quote for Top Channel Letters Inc [1a016973e6aeb99e]
+Tue, 18 Aug 2026 15:16:17 -0500: Request a Bond of Bridgeview [1a01684757b82c05]</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
         <is>
           <t>Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609 www
-Thank you for the quote request with BondExchange, the surety partner of Karstens Financial LLC. You are approved for the following bond quote: $10000 IL License/Permit bond Bond Term Cost Due Now</t>
+Thank you for the quote request with BondExchange, the surety partner of Karstens Financial LLC. You are approved for the following bond quote: $10000 IL License/Permit bond Bond Term Cost Due Now
+Hi, Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609</t>
         </is>
       </c>
     </row>
@@ -13597,19 +13610,21 @@
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>Sun, 16 Aug 2026 18:53:31 -0500</t>
+          <t>Tue, 18 Aug 2026 16:08:05 -0500</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
           <t>Wed, 12 Aug 2026 13:32:23 -0500: Re: RFQ - "FASTSIGNS" sign [19ff73fbf1f11591]
-Sun, 16 Aug 2026 18:53:31 -0500: Re: RFQ - "FASTSIGNS" sign [1a00cfea99cd6084]</t>
+Sun, 16 Aug 2026 18:53:31 -0500: Re: RFQ - "FASTSIGNS" sign [1a00cfea99cd6084]
+Tue, 18 Aug 2026 16:08:05 -0500: Re: RFQ - "FASTSIGNS" sign [1a016b3eabb1ab55]</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
           <t>Yes. This color will work. Ravi. On Wed, Aug 12, 2026 at 11:46 AM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi Ravi, Please see attached photo PMS 427 C and the color we have in the sign
-Finally we got the vinyl . There is still a problem with the supplier , they sent us a 48&amp;quot;x50yards roll .crazy.! I will have this job completed very soon. do not remember if you need us to install</t>
+Finally we got the vinyl . There is still a problem with the supplier , they sent us a 48&amp;quot;x50yards roll .crazy.! I will have this job completed very soon. do not remember if you need us to install
+Buddy, The sign is ready for pick up! please see photos in attachment. our address is 1111 w 35th street .let us know when you will come.so we can have that ready for you! Thanks again for you trust!</t>
         </is>
       </c>
     </row>
@@ -14515,7 +14530,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -14540,19 +14555,21 @@
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Sun, 16 Aug 2026 23:02:52 -0500</t>
+          <t>Tue, 18 Aug 2026 22:42:40 +0000</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
           <t>Fri, 14 Aug 2026 17:01:14 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0024b5160293ad]
-Sun, 16 Aug 2026 23:02:52 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a00de2eea056286]</t>
+Sun, 16 Aug 2026 23:02:52 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a00de2eea056286]
+Tue, 18 Aug 2026 22:42:40 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0170b0c263cade]</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
         <is>
           <t>Hello Charles, I am in the process of opening a new Stretch Zone studio at 1733 W. Kirby Avenue in Champaign and would like to request a proposal for the fabrication and installation of our exterior
-Hi, is this sport clip your shop? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W</t>
+Hi, is this sport clip your shop? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W
+Hi Lowa, I have requested of Landlord&amp;#39;s broker any exterior elevations they may have for reference. Your signage is a great investment for your business. This pursuit is the tenant&amp;#39;s own with</t>
         </is>
       </c>
     </row>
@@ -14611,7 +14628,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -14636,17 +14653,21 @@
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 18:58:12 +0000</t>
+          <t>Tue, 18 Aug 2026 17:17:47 +0000</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 18:58:12 +0000: Sign Review - Woodfield Mall/Digiso (resubmit) [1a001a3b71eda616]</t>
+          <t>Fri, 14 Aug 2026 18:58:12 +0000: Sign Review - Woodfield Mall/Digiso (resubmit) [1a001a3b71eda616]
+Tue, 18 Aug 2026 12:18:49 -0500: Fwd: Sign Review - Woodfield Mall/Digiso (resubmit) [1a015e1f9c4ce607]
+Tue, 18 Aug 2026 17:17:47 +0000: Automatic reply: [EXT] Re: Sign Review - Woodfield Mall/Digiso (resubmit) [1a015e11d58bc2ee]</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t>Attached please find a review letter and drawings. Please direct questions to Sam Felling regarding the review. Thanks Stephanie Allen Senior Analyst Tenant Coordination The Simon® logo consisting of a</t>
+          <t>Attached please find a review letter and drawings. Please direct questions to Sam Felling regarding the review. Thanks Stephanie Allen Senior Analyst Tenant Coordination The Simon® logo consisting of a
+Hi, Samantha and Stephanie Thank you for reviewing. Attached is the revised Sign Rendering according to the letter you sent Please check and let us know if anything needs to change. Thank you so much
+Hello-I am out of the office this afternoon, Tuesday 8/18. If an urgent plan/sign issue, please reach out to simontctenantplans@simon.com, otherwise I will respond to your email when I return. Thanks!</t>
         </is>
       </c>
     </row>
@@ -15085,7 +15106,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -15110,17 +15131,19 @@
       </c>
       <c r="K311" t="inlineStr">
         <is>
-          <t>Mon, 17 Aug 2026 19:26:34 +0000</t>
+          <t>Tue, 18 Aug 2026 20:29:43 +0000</t>
         </is>
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>Mon, 17 Aug 2026 19:26:34 +0000: Interior illuminated sign [1a01130b8f9cdfdc]</t>
+          <t>Mon, 17 Aug 2026 19:26:34 +0000: Interior illuminated sign [1a01130b8f9cdfdc]
+Tue, 18 Aug 2026 20:29:43 +0000: Re: Interior illuminated sign [1a01690ebb03ffc5]</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
         <is>
-          <t>Hi Charles, Could you please provide a production quote for an interior illuminated sign? A few details: Interior sign Back-lit / halo-lit No installation required, production only Approximate size: 18</t>
+          <t>Hi Charles, Could you please provide a production quote for an interior illuminated sign? A few details: Interior sign Back-lit / halo-lit No installation required, production only Approximate size: 18
+Hi Charles, Thank you for the quote. We have one more project we&amp;#39;d like quoted. Could you please provide pricing for the production and installation of channel letters? The size and layout are</t>
         </is>
       </c>
     </row>
@@ -15638,6 +15661,852 @@
       <c r="M322" t="inlineStr">
         <is>
           <t>1. 圆形灯箱 55&amp;#39;&amp;#39; 2. SHINTO 80.5&amp;#39;&amp;#39;x26.5&amp;#39;&amp;#39; 3. JAPANESE STEAKHOUSE &amp;amp; SUSHI 228&amp;#39;&amp;#39;x13&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-0322</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Presotea - Sign Info Re: Presotea - Sign Info Re: Presotea - Sign Info Re: Presotea - Sign Info</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>tony.liu@presoteacorporation.com</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 16:58:24 -0500</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 16:58:24 -0500: Re: Presotea - Sign Info [1a016e28e1453211]</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>Hi Charles, Thanks for your reply with the info! We will have to actually measure them and send you. Many thanks. Great days. Best, Tony Sent from my iPhone On Aug 17, 2026, at 5:54 PM, charles zhao</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-0323</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Inspection Report (Sign Inspection) for Inspection: Sign Inspection</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>cityview_donotreply@downers.us</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>18 Aug 2026 16:17:35 -0400</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>18 Aug 2026 16:17:35 -0400: Inspection Report (Sign Inspection) for Inspection: Sign Inspection [1a01685b16ebd264]</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>The attached letter has been sent to you by the Village of Downers Grove. Attached Document: Inspection Report (Sign Inspection) Inspection: Sign Inspection Outcome: Passed Permit Number: 24-PSG-0031</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-0324</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Only) Auto Zone Sign</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 13:03:58 -0700</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 13:03:58 -0700: (Estimate Only) Auto Zone Sign [1a016796ca3e338d]</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>客人提供的文件实际尺寸 Sign 1 496&amp;#39;&amp;#39;x50.8&amp;#39;&amp;#39; Sign2 496&amp;#39;&amp;#39;x 48.77&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-0325</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Sign Renderings – Landlord Approval Request</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Pylon Sign</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>shikibuffet6249@gmail.com</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 14:36:15 -0500</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 14:36:15 -0500: Re: Sign Renderings – Landlord Approval Request [1a0166007b1f364c]</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>Hi, TCP Please see the property management comment below regarding the pylon sign. Can you please follow up. On Mon, Aug 17, 2026 at 21:49 Vera Putro &amp;lt;vera@xroadsadvisors.com&amp;gt; wrote: Hi Julien -</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-0326</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>AutoZone</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>george@pdichi.com</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 19:19:00 +0000</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 19:19:00 +0000: AutoZone [1a016502ed9543fd]</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>Charles! Please Quote George H. Ramirez Direct: (224) 432 - 9191 George@pdichi.com | www.PDICHI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-0327</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Welcome to MailerLite!</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>info@mailerlite.com</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>18 Aug 2026 18:30:27 -0000</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>18 Aug 2026 18:30:27 -0000: Welcome to MailerLite! [1a01623a2651bcd8]</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>Here&amp;#39;s how to get started with your account View in browser Log in Welcome to MailerLite! Hi there, We&amp;#39;re super excited you joined the MailerLite family 🎉. Let&amp;#39;s begin your 14-day trial</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-0328</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Dumpling Pub 灯箱片 Production File (J)</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 11:10:50 -0700</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 11:10:50 -0700: Dumpling Pub 灯箱片 Production File (J) [1a01611dbe50fb16]</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>实际完成尺寸 95.625&amp;#39;&amp;#39; x 29.875&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-0329</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>American Sign - Pure Medical Spa (Skokie) Production File (J)</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 10:44:23 -0700</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 10:44:23 -0700: American Sign - Pure Medical Spa (Skokie) Production File (J) [1a015f9b912b09dd]</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>黑色return,黑色trim cap。黑白膜的面。 raceway待定。 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-0330</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Mayor's Storm Update - 8.18.2026 - 12 p.m.</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>admin@public.govdelivery.com</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 17:01:38 +0000</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 17:01:38 +0000: Mayor's Storm Update - 8.18.2026 - 12 p.m. [1a015d24cb688c4a]</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>Having trouble viewing this email? View it as a Web page. | Bookmark and Share SUBSCRIBER SERVICES Manage Subscriptions | Unsubscribe | Help Neighbors, The severe weather we have experienced this</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-0331</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Landlord Approval Needed for Red Crab， 4901 WASHINGTON AVE, RACINE, WI 53406</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>pat@signatureteamrealtors.com</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 11:54:40 -0500</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 11:54:40 -0500: Landlord Approval Needed for Red Crab， 4901 WASHINGTON AVE, RACINE, WI 53406 [1a015cbe16906dc9]</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>Dear Landlord, This is Top Channel Letter, we are the sign contractor for your tenant Red Crab Juicy seafood Bar, located in 4901 WASHINGTON AVE, RACINE, WI 53406 Please review the attached plans and</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-0332</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Your Toyota Sienna held its estimated value!</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>donotreply@mail.carvana.com</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 16:51:03 +0000</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 16:51:03 +0000: Your Toyota Sienna held its estimated value! [1a015c89ee4e4a6d]</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>A steady estimated value can be a good time to sell. ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-0333</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Website Temporarily Unavailable</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>encompass-more</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 12:49:43 -0400 (EDT)</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 12:49:43 -0400 (EDT): Website Temporarily Unavailable [1a015c761e354f2d]</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>Sorry for any inconvenience! Get FREE Shipping on orders of $300 or more! *Purchase must be under 25lb My Account Login sales@encompass-more.com Questions? Toll Free: (855) 286-3368 Facebook Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-0334</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Thank You for Registering for the 2026 Midwest Sign and Graphics Show, Chicago!</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>tyhull@wensco.com</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 12:21:02 -0400</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 12:21:02 -0400: Thank You for Registering for the 2026 Midwest Sign and Graphics Show, Chicago! [1a015ad1ffab841b]</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>Click to add to your calendar! ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏ ͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-0335</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>New sign-in to your Shopify account</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>mailer@shopify.com</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 16:08:36 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 16:08:36 +0000 (UTC): New sign-in to your Shopify account [1a015a1bd15e1679]</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>August 18, 2026 New device signed in Review activity We noticed a new sign-in to your account from a new device. If this was you, you&amp;#39;re all set — no action needed. Device: Chrome 151 on Windows 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-0336</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Pure Medical Spa Skokie Re: Pure Medical Spa Skokie Re: Pure Medical Spa Skokie Re: Pure Medical Spa Skokie Re: Pure Med</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>abid@americansign.us</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 10:33:22 -0500</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Tue, 18 Aug 2026 10:33:22 -0500: Re: Pure Medical Spa Skokie [1a015817a1e20a26]</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>black trim cap . black return . Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-0337</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Tidal Thai Sign Production File</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 16:12:03 -0700</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 16:12:03 -0700: Tidal Thai Sign Production File [1a011ff451757914]</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>大陆生产 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-0338</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Possible Inquiry Re: Possible Inquiry</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>signarama joliet</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 14:18:34 +0000</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Mon, 17 Aug 2026 14:18:34 +0000: Re: Possible Inquiry [1a01016bb42b4f48]</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>I will give you a call today when I get a chance. Just so you know there is nothing to remove, installation only. So just to clarify it would be $2200 Installed + permit fees of $250 for a total of</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-0339</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Sign Proposal and Installation Agreement</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>dhurley580@aol.com</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 22:21:16 -0500</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Sun, 16 Aug 2026 22:21:16 -0500: Re: Sign Proposal and Installation Agreement [1a00dbcdabb711c5]</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>Dear Donald, Thanks for your reply. we will talk to the business owner and start production Thanks! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-19
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M340"/>
+  <dimension ref="A1:M364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -9724,17 +9724,19 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Thu, 23 Jul 2026 21:00:27 +0800 (GMT+08:00)</t>
+          <t>Wed, 19 Aug 2026 17:35:12 +0000 (UTC)</t>
         </is>
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>Thu, 23 Jul 2026 21:00:27 +0800 (GMT+08:00): RFQ Signage project [19f8f10abaaff1e2]</t>
+          <t>Thu, 23 Jul 2026 21:00:27 +0800 (GMT+08:00): RFQ Signage project [19f8f10abaaff1e2]
+Wed, 19 Aug 2026 17:35:12 +0000 (UTC): Brown Beagle Sign: From Concept to Completion [1a01b176535500af]</t>
         </is>
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>Dear Sir, I&amp;#39;m Bryan, Director of SUN SIGN in China. Do you provide Signage for Restaurants, Retail stores, Chain brand, exhibitions, and hotels? We are your outsourcing company with Design,</t>
+          <t>Dear Sir, I&amp;#39;m Bryan, Director of SUN SIGN in China. Do you provide Signage for Restaurants, Retail stores, Chain brand, exhibitions, and hotels? We are your outsourcing company with Design,
+When a sign shop needed a detailed design for a new industrial park sign, Easelly helped bring the concept for Brown Beagle Industrial Park to life. ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌ ‌</t>
         </is>
       </c>
     </row>
@@ -9971,7 +9973,8 @@
 Fri, 14 Aug 2026 12:59:19 +0000: RE: Policies [1a0005b0c286f06f]
 Tue, 18 Aug 2026 16:29:20 -0500: Life Space Digital Invoice &amp; COI from Top Channel Letters [1a016c764718db5d]
 Tue, 18 Aug 2026 16:13:42 -0500: Fwd: coi [1a016b94677bc643]
-Tue, 18 Aug 2026 15:59:01 -0500: Fwd: coi [1a016abd350fc6d3]</t>
+Tue, 18 Aug 2026 15:59:01 -0500: Fwd: coi [1a016abd350fc6d3]
+Wed, 19 Aug 2026 14:42:46 +0000: Fw: Life Space Digital Invoice &amp; COI from Top Channel Letters [1a01a7998855bb61]</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -9982,7 +9985,8 @@
 Please call 219 755 3730. This is the number to our recorder&amp;#39;s office. They aren&amp;#39;t even located within the same town as me. They should be able to help you. From: charles zhao &amp;lt;
 Dear Sunny, Please see attached invoice and COI. Feel free to contact us if you have any questions. Thank you! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:
 ---------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 4:10 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan
----------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 3:53 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan</t>
+---------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 3:53 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan
+Hi Charles and Candy, Well received the proposal and the COI, we will confirm with you once we received approval from the building. Sunny Chen Head of Operations M: 347.993.9116 lifespacedigital.com</t>
         </is>
       </c>
     </row>
@@ -10028,14 +10032,17 @@
 Thu, 13 Aug 2026 17:04:56 -0500: Re: Right of Way Bond/Surety Bond  needed for Village of La Grange, IL [19ffd28295f9fb54]
 Fri, 14 Aug 2026 16:09:45 -0400: Bond Quote for Top Channel Letters Inc [1a001e51ba1b2a17]
 Tue, 18 Aug 2026 16:36:45 -0400: Bond Quote for Top Channel Letters Inc [1a016973e6aeb99e]
-Tue, 18 Aug 2026 15:16:17 -0500: Request a Bond of Bridgeview [1a01684757b82c05]</t>
+Tue, 18 Aug 2026 15:16:17 -0500: Request a Bond of Bridgeview [1a01684757b82c05]
+Wed, 19 Aug 2026 12:27:27 -0500: Re: Quote #784591 – Unable to Upload Sign Agreement [1a01b1074dc49453]
+Wed, 19 Aug 2026 13:12:30 -0400: Bond Quote for Top Channel Letters Inc [1a01b02a6e71aed9]</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
         <is>
           <t>Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609 www
 Thank you for the quote request with BondExchange, the surety partner of Karstens Financial LLC. You are approved for the following bond quote: $10000 IL License/Permit bond Bond Term Cost Due Now
-Hi, Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609</t>
+Hi, Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609
+Hello Charles, Yes, you can send the signed agreement to us and we can upload and process everythingon ourselves. Thanks, On Wed, Aug 19, 2026 at 12:10 PM charles zhao &amp;lt;topchannelletters@gmail.com</t>
         </is>
       </c>
     </row>
@@ -11944,21 +11951,23 @@
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 16:19:24 -0500</t>
+          <t>Tue, 18 Aug 2026 10:07:05 -0500</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
         <is>
           <t>Tue, 21 Jul 2026 14:25:16 -0500: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [19f8623b9f970dab]
 Fri, 14 Aug 2026 16:19:24 -0500: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a00224d432e9243]
-Mon, 17 Aug 2026 21:22:12 +0000: RE: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a0119a9d601f480]</t>
+Mon, 17 Aug 2026 21:22:12 +0000: RE: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a0119a9d601f480]
+Tue, 18 Aug 2026 10:07:05 -0500: Re: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a015695e8912f87]</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
           <t>Hi, Martin We are Top Channel Letters, the sign contractor for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 We would like to apply for a sign permit for this business. The attachments include
 Hi, Lisa This is the revision for sign 3, we have updated a smaller sign to fit the requirement. Please check. Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top
-Good Afternoon, Please refer to the attached letter that our Chief Building Inspector, Ray Graefen sent regarding the review your signs. We are still in need of a response letter with electrical</t>
+Good Afternoon, Please refer to the attached letter that our Chief Building Inspector, Ray Graefen sent regarding the review your signs. We are still in need of a response letter with electrical
+got it, thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St</t>
         </is>
       </c>
     </row>
@@ -13585,7 +13594,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -13610,21 +13619,23 @@
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 16:08:05 -0500</t>
+          <t>Wed, 19 Aug 2026 10:32:37 -0500</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
           <t>Wed, 12 Aug 2026 13:32:23 -0500: Re: RFQ - "FASTSIGNS" sign [19ff73fbf1f11591]
 Sun, 16 Aug 2026 18:53:31 -0500: Re: RFQ - "FASTSIGNS" sign [1a00cfea99cd6084]
-Tue, 18 Aug 2026 16:08:05 -0500: Re: RFQ - "FASTSIGNS" sign [1a016b3eabb1ab55]</t>
+Tue, 18 Aug 2026 16:08:05 -0500: Re: RFQ - "FASTSIGNS" sign [1a016b3eabb1ab55]
+Wed, 19 Aug 2026 10:32:37 -0500: Re: RFQ - "FASTSIGNS" sign [1a01aa75357c15fd]</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
           <t>Yes. This color will work. Ravi. On Wed, Aug 12, 2026 at 11:46 AM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi Ravi, Please see attached photo PMS 427 C and the color we have in the sign
 Finally we got the vinyl . There is still a problem with the supplier , they sent us a 48&amp;quot;x50yards roll .crazy.! I will have this job completed very soon. do not remember if you need us to install
-Buddy, The sign is ready for pick up! please see photos in attachment. our address is 1111 w 35th street .let us know when you will come.so we can have that ready for you! Thanks again for you trust!</t>
+Buddy, The sign is ready for pick up! please see photos in attachment. our address is 1111 w 35th street .let us know when you will come.so we can have that ready for you! Thanks again for you trust!
+i would say $120 for delivery Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St</t>
         </is>
       </c>
     </row>
@@ -13661,17 +13672,20 @@
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 13:36:14 -0400 (EDT)</t>
+          <t>Wed, 19 Aug 2026 06:39:36 -0700</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>Wed, 12 Aug 2026 13:36:14 -0400 (EDT): IMPORTANT INFORMATION [19ff70bf368a59a4]</t>
+          <t>Wed, 12 Aug 2026 13:36:14 -0400 (EDT): IMPORTANT INFORMATION [19ff70bf368a59a4]
+Wed, 19 Aug 2026 12:58:48 -0700: IMPORTANT INFORMATION [1a01b9adfa48c046]
+Wed, 19 Aug 2026 06:39:36 -0700: IMPORTANT INFORMATION [1a01a3fbfbedf40f]</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>You have a secure message, please view details below. CITY OF NAPERVILLE UPDATE BUILDING PERMIT CONTRACTORS UPDATE Address: 400 S. Eagle Street Naperville, IL 60540 https://www.naperville.il.us/</t>
+          <t>You have a secure message, please view details below. CITY OF NAPERVILLE UPDATE BUILDING PERMIT CONTRACTORS UPDATE Address: 400 S. Eagle Street Naperville, IL 60540 https://www.naperville.il.us/
+Secure Message Secure Message You have a secure message Please view details below. CITY OF NAPERVILLE — update View Message Address 400 S. Eagle Street Naperville, IL 60540 This is an automated</t>
         </is>
       </c>
     </row>
@@ -14037,17 +14051,19 @@
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>Thu, 13 Aug 2026 16:34:20 -0500</t>
+          <t>Wed, 19 Aug 2026 16:08:54 +0000</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>Thu, 13 Aug 2026 16:34:20 -0500: Re: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [19ffd0c26e0fffd5]</t>
+          <t>Thu, 13 Aug 2026 16:34:20 -0500: Re: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [19ffd0c26e0fffd5]
+Wed, 19 Aug 2026 16:08:54 +0000: RE: Regarding Canopy Sign Permit / UDC Approval – 3313 University Ave [1a01ac877eaafd3d]</t>
         </is>
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Hi, Jessica Sorry for late response Would you and Chrissy still available on Tuesday, August 18 at 11 AM, 1:30 PM, 2:30 PM Thank you for assistance Best Regards, Charles Zhao Top Channel Letters Top</t>
+          <t>Hi, Jessica Sorry for late response Would you and Chrissy still available on Tuesday, August 18 at 11 AM, 1:30 PM, 2:30 PM Thank you for assistance Best Regards, Charles Zhao Top Channel Letters Top
+Please fine attached the site plan we have on file for you to use for the awning submittal. Chrissy Thiele Zoning Inspector City of Madison Building Inspection Division 215 Martin Luther King Jr. Blvd</t>
         </is>
       </c>
     </row>
@@ -14555,21 +14571,23 @@
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 22:42:40 +0000</t>
+          <t>Wed, 19 Aug 2026 18:22:51 +0000</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
           <t>Fri, 14 Aug 2026 17:01:14 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0024b5160293ad]
 Sun, 16 Aug 2026 23:02:52 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a00de2eea056286]
-Tue, 18 Aug 2026 22:42:40 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0170b0c263cade]</t>
+Tue, 18 Aug 2026 22:42:40 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0170b0c263cade]
+Wed, 19 Aug 2026 18:22:51 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a01b4377a1ae38c]</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
         <is>
           <t>Hello Charles, I am in the process of opening a new Stretch Zone studio at 1733 W. Kirby Avenue in Champaign and would like to request a proposal for the fabrication and installation of our exterior
 Hi, is this sport clip your shop? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W
-Hi Lowa, I have requested of Landlord&amp;#39;s broker any exterior elevations they may have for reference. Your signage is a great investment for your business. This pursuit is the tenant&amp;#39;s own with</t>
+Hi Lowa, I have requested of Landlord&amp;#39;s broker any exterior elevations they may have for reference. Your signage is a great investment for your business. This pursuit is the tenant&amp;#39;s own with
+Hi Lowa, Landlord nor its broker have any elevation drawings for reference nor prior signage exhibits on this space in Old Farm. Your signage renderings will all have to be drawn up from the pictures/</t>
         </is>
       </c>
     </row>
@@ -14660,14 +14678,16 @@
         <is>
           <t>Fri, 14 Aug 2026 18:58:12 +0000: Sign Review - Woodfield Mall/Digiso (resubmit) [1a001a3b71eda616]
 Tue, 18 Aug 2026 12:18:49 -0500: Fwd: Sign Review - Woodfield Mall/Digiso (resubmit) [1a015e1f9c4ce607]
-Tue, 18 Aug 2026 17:17:47 +0000: Automatic reply: [EXT] Re: Sign Review - Woodfield Mall/Digiso (resubmit) [1a015e11d58bc2ee]</t>
+Tue, 18 Aug 2026 17:17:47 +0000: Automatic reply: [EXT] Re: Sign Review - Woodfield Mall/Digiso (resubmit) [1a015e11d58bc2ee]
+Wed, 19 Aug 2026 15:07:13 +0000: Re: [EXT] Fwd: Sign Review - Woodfield Mall/Digiso (resubmit) [1a01a8ff3047d035]</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
         <is>
           <t>Attached please find a review letter and drawings. Please direct questions to Sam Felling regarding the review. Thanks Stephanie Allen Senior Analyst Tenant Coordination The Simon® logo consisting of a
 Hi, Samantha and Stephanie Thank you for reviewing. Attached is the revised Sign Rendering according to the letter you sent Please check and let us know if anything needs to change. Thank you so much
-Hello-I am out of the office this afternoon, Tuesday 8/18. If an urgent plan/sign issue, please reach out to simontctenantplans@simon.com, otherwise I will respond to your email when I return. Thanks!</t>
+Hello-I am out of the office this afternoon, Tuesday 8/18. If an urgent plan/sign issue, please reach out to simontctenantplans@simon.com, otherwise I will respond to your email when I return. Thanks!
+Hi Charles, Raceways like this are not permitted. Is there another way to attach the letters? Sammy Felling Tenant Coordinator Tenant Coordination The Simon® logo consisting of a double-diamond design</t>
         </is>
       </c>
     </row>
@@ -14753,19 +14773,21 @@
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>Mon, 17 Aug 2026 12:28:53 +0000</t>
+          <t>Wed, 19 Aug 2026 11:49:49 -0500</t>
         </is>
       </c>
       <c r="L303" t="inlineStr">
         <is>
           <t>Fri, 14 Aug 2026 12:47:14 -0500: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a00162959aa0e3e]
-Mon, 17 Aug 2026 12:28:53 +0000: RE: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a00fb258a5a2c48]</t>
+Mon, 17 Aug 2026 12:28:53 +0000: RE: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a00fb258a5a2c48]
+Wed, 19 Aug 2026 11:49:49 -0500: Re: Sign Application for Nori Sushi &amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 [1a01aedc82df3dce]</t>
         </is>
       </c>
       <c r="M303" t="inlineStr">
         <is>
           <t>Dear Town Hall, We are Top Channel Letters, the sign contractor for Nori Sushi &amp;amp; Grill, N 162, Eisenhower Dr, Appleton, WI 54915 We would like to apply for a sign permit for this business. The
-Hi Charles ~ Thank you for this information! I apologize, but the form you filled out for a sign request pertains to our sign out front, if residents want to put something on our sign (I can see the</t>
+Hi Charles ~ Thank you for this information! I apologize, but the form you filled out for a sign request pertains to our sign out front, if residents want to put something on our sign (I can see the
+Hi Tina, Thank you so much for the clarification and the link. I will get the General Building Permit filled out and reply to all as requested. Best regards, Charles Zhao Best Regards, Charles Zhao Top</t>
         </is>
       </c>
     </row>
@@ -16026,17 +16048,19 @@
       </c>
       <c r="K330" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 10:44:23 -0700</t>
+          <t>Wed, 19 Aug 2026 12:24:12 -0500</t>
         </is>
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 10:44:23 -0700: American Sign - Pure Medical Spa (Skokie) Production File (J) [1a015f9b912b09dd]</t>
+          <t>Tue, 18 Aug 2026 10:44:23 -0700: American Sign - Pure Medical Spa (Skokie) Production File (J) [1a015f9b912b09dd]
+Wed, 19 Aug 2026 12:24:12 -0500: Re: American Sign - Pure Medical Spa (Skokie) Production File (J) [1a01b0d837c031e0]</t>
         </is>
       </c>
       <c r="M330" t="inlineStr">
         <is>
-          <t>黑色return,黑色trim cap。黑白膜的面。 raceway待定。 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.</t>
+          <t>黑色return,黑色trim cap。黑白膜的面。 raceway待定。 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.
+white raceway 白色！ On Tue, Aug 18, 2026 at 12:44 PM Qa Prints &amp;lt;info.qaprints@gmail.com&amp;gt; wrote: 黑色return,黑色trim cap。黑白膜的面。 raceway待定。 Best Regards, Charles Zhao QaPrints Best Price for large</t>
         </is>
       </c>
     </row>
@@ -16449,17 +16473,19 @@
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>Mon, 17 Aug 2026 14:18:34 +0000</t>
+          <t>Wed, 19 Aug 2026 19:31:31 +0000</t>
         </is>
       </c>
       <c r="L339" t="inlineStr">
         <is>
-          <t>Mon, 17 Aug 2026 14:18:34 +0000: Re: Possible Inquiry [1a01016bb42b4f48]</t>
+          <t>Mon, 17 Aug 2026 14:18:34 +0000: Re: Possible Inquiry [1a01016bb42b4f48]
+Wed, 19 Aug 2026 19:31:31 +0000: Re: Possible Inquiry [1a01b820cb36f9df]</t>
         </is>
       </c>
       <c r="M339" t="inlineStr">
         <is>
-          <t>I will give you a call today when I get a chance. Just so you know there is nothing to remove, installation only. So just to clarify it would be $2200 Installed + permit fees of $250 for a total of</t>
+          <t>I will give you a call today when I get a chance. Just so you know there is nothing to remove, installation only. So just to clarify it would be $2200 Installed + permit fees of $250 for a total of
+Sorry I have not gotten a chance to call yet Charles, I will call soon later today. I have sent over another proof for more channel letters. The exact same type of channel letters as the previous</t>
         </is>
       </c>
     </row>
@@ -16507,6 +16533,1134 @@
       <c r="M340" t="inlineStr">
         <is>
           <t>Dear Donald, Thanks for your reply. we will talk to the business owner and start production Thanks! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-0340</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Landloard Approval Needed for Ou's Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>tfshank@aol.com</t>
+        </is>
+      </c>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:29:21 -0500</t>
+        </is>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:29:21 -0500: Landloard Approval Needed for Ou's Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 [1a01c24a35502c2b]</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>Dear Landlord, This is Top Channel Letters, we are the sign contractor for your tenant Ou&amp;#39;s Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 Please see attached, you will find the</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-0341</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Pure Medical Spa Lightbox Sign Production File(J)</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Cabinet Sign</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 15:27:15 -0700</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 15:27:15 -0700: Pure Medical Spa Lightbox Sign Production File(J) [1a01c2305f203d3b]</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>48“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St,</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-0342</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>(order)pure light box 48" single side Re: (order)pure light box 48" single side Re: (order)pure light box 48" single sid</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>abid@americansign.us</t>
+        </is>
+      </c>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:18:07 -0500</t>
+        </is>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:18:07 -0500: Re: (order)pure light box 48" single side [1a01c1a9c2d2f43c]</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>Is this translucent pink? Yes need switch, confirmed Sent from my iPhone On Aug 19, 2026, at 4:55 PM, charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: ﻿ we have this pink Best Regards, Charles</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-0343</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Baum Realty Group</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>zach@baumrealty.com</t>
+        </is>
+      </c>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:16:08 -0500</t>
+        </is>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:16:08 -0500: Partnership Proposal | Preferred Signage Program for Baum Realty Group [1a01be1a8a3b2cf1]</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-0344</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for CBRE</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>joe.parrott@cbre.com</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:16:06 -0500</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:16:06 -0500: Partnership Proposal | Preferred Signage Program for CBRE [1a01be1a15743625]</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-0345</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Baum Realty Group</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>paul@baumrealty.com</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:16:03 -0500</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:16:03 -0500: Partnership Proposal | Preferred Signage Program for Baum Realty Group [1a01be196f1bbd7d]</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-0346</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Baum Realty Group</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>keving@baumrealty.com</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:58 -0500</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:58 -0500: Partnership Proposal | Preferred Signage Program for Baum Realty Group [1a01be18393f84c4]</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-0347</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Harrison Properties</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>tberlinghof@hpre.com</t>
+        </is>
+      </c>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:54 -0500</t>
+        </is>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:54 -0500: Partnership Proposal | Preferred Signage Program for Harrison Properties [1a01be170953074e]</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-0348</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Baum Realty Group</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>doug.renner@baumrealty.com</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:51 -0500</t>
+        </is>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:51 -0500: Partnership Proposal | Preferred Signage Program for Baum Realty Group [1a01be166d3733c9]</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-0349</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Tucker Development</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>klawson@tuckerdevelopment.com</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:27 -0500</t>
+        </is>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:27 -0500: Partnership Proposal | Preferred Signage Program for Tucker Development [1a01be106c6100e8]</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-0350</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Mid-America Asset Management</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>cwickland@midamericagrp.com</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:22 -0500</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:22 -0500: Partnership Proposal | Preferred Signage Program for Mid-America Asset Management [1a01be0f5efae5e8]</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-0351</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Partnership Proposal | Preferred Signage Program for Mid-America Asset Management</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>mgraham@midamericagrp.com</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:19 -0500</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:19 -0500: Partnership Proposal | Preferred Signage Program for Mid-America Asset Management [1a01be0e8ded567d]</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-0352</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From TopChannelLetters</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>sean.mccourt@cbre.com</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:15 -0500</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 16:15:15 -0500: Partnership Proposal From TopChannelLetters [1a01be0d96964497]</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>A preferred signage partnership for more consistent properties, a simpler tenant path, and program benefits tied to completed work. Top Channel Letters Chicago Fabrication Facility Partner Proposal For</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-0353</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>A Pizza Quote</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>george@pdichi.com</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 20:40:38 +0000</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 20:40:38 +0000: A Pizza Quote [1a01bc147aa74a08]</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>Charles No Led No Paint raceway White 3/4&amp;quot; Trim cap White Returns 3&amp;quot; or whatever easier We pay and pick up 2 Weeks $2300? George H. Ramirez Direct: (224) 432 - 9191 George@pdichi.com | www.</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-0354</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Halo lit acrylic back channel letter with chrome finish Re: Halo lit acrylic back channel letter with chrome finish</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>mike@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 14:24:27 -0500</t>
+        </is>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 14:24:27 -0500: Re: Halo lit acrylic back channel letter with chrome finish [1a01b7b6c7543d45]</t>
+        </is>
+      </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>Hi, Thank you for contacting us, we are working on it now, will get back to you soon. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-0355</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Welcome to Cloudinary! - Get started in minutes</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>digital-cs@cloudinary.com</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 19:07:17 +0000</t>
+        </is>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 19:07:17 +0000: Welcome to Cloudinary! - Get started in minutes [1a01b6bb4ce03f89]</t>
+        </is>
+      </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>Hi charles, Welcome to Cloudinary 👋 — the fastest way to manage and optimize your media at scale. Let&amp;#39;s start by connecting to Cloudinary: Coding with AI: Try the AI Powerstart Get your API keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-0356</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Fw: New Website Inquiry | Laboy Pawn &amp; Gold | ID:1986085 Re: Fw: New Website Inquiry | Laboy Pawn &amp; Gold | ID:1986085</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>signarama woodridge</t>
+        </is>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 18:18:39 +0000</t>
+        </is>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 18:18:39 +0000: Re: Fw: New Website Inquiry | Laboy Pawn &amp; Gold | ID:1986085 [1a01b3f45a29d1ba]</t>
+        </is>
+      </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>Hi Charles, We&amp;#39;re moving forward with the Laboy Pawn &amp;amp; Gold project and wanted to check if the pricing you previously provided is still good for this job. We will not be needing installation</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-0357</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Interior illuminated sign Re: Interior illuminated sign Re: Interior illuminated sign Re: Interior illuminated sign</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>signarama woodridge</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:47:01 +0000</t>
+        </is>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:47:01 +0000: Re: Interior illuminated sign [1a01b223c0d3440b]</t>
+        </is>
+      </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>It should be this size and a raceway would need to be produced as well. Thanks! From: charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Tuesday, August 18, 2026 4:04 PM To: Signarama Woodridge, IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-0358</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Payment Awaiting</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Wensco Sign Supply - Invoice# 4025905</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>ar@wensco.com</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 13:03:10 -0400</t>
+        </is>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 13:03:10 -0400: Wensco Sign Supply - Invoice# 4025905 [1a01afa2cb8fbfc1]</t>
+        </is>
+      </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>Billing Contact TOP CHANNEL LETTERS INC See attached file(s). Kay James Wensco Sign Supply ar@wensco.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-0359</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>(mk chicken canopy size) Hana Awning OTP</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Awning</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 11:27:37 -0500</t>
+        </is>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 11:27:37 -0500: Fwd: (mk chicken canopy size) Hana Awning OTP [1a01ad9b6fdcc363]</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com ---------- Forwarded message -</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-0360</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Savvy Sliders Re: FW: Savvy Sliders</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>aaron@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 11:17:54 -0500</t>
+        </is>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 11:17:54 -0500: Re: FW: Savvy Sliders [1a01ad09c47b51a7]</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>give me a call bro Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL,</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-0361</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Presotea - Sign Info Re: Presotea - Sign Info</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>tony.liu@presoteacorporation.com</t>
+        </is>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 10:44:33 -0500</t>
+        </is>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 10:44:33 -0500: Re: Presotea - Sign Info [1a01ab20de8d3f82]</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>Can You give me a call when you have time? my number is 3124042130. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-0362</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Correspondence from Village of Downers Grove - Permit Approval Notice (26-PSG-0039)</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>cityview_donotreply@downers.us</t>
+        </is>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>19 Aug 2026 09:35:19 -0400</t>
+        </is>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>19 Aug 2026 09:35:19 -0400: Correspondence from Village of Downers Grove - Permit Approval Notice (26-PSG-0039) [1a01a3bc7c45afec]</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>Please see attached document. This email was sent from Downers Grove Production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-0363</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Is your store still waiting to be built?</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>email@email.shopify.com</t>
+        </is>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 09:46:08 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 09:46:08 +0000 (UTC): Is your store still waiting to be built? [1a01969f5347512d]</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>You could get up to $10000 back in credits ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-20
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M364"/>
+  <dimension ref="A1:M392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -957,7 +957,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 10:52:03 +0700</t>
+          <t>Thu, 20 Aug 2026 10:20:59 +0700</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -965,7 +965,8 @@
           <t>Tue, 11 Aug 2026 22:31:20 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ff1734a1184586]
 Thu, 13 Aug 2026 11:15:30 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [19ffbe84b6b9d8a3]
 Sun, 16 Aug 2026 22:28:29 -0500: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a00dc37655eb712]
-Tue, 18 Aug 2026 10:52:03 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a012ff9cfedabf7]</t>
+Tue, 18 Aug 2026 10:52:03 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a012ff9cfedabf7]
+Thu, 20 Aug 2026 10:20:59 +0700: Re: Landlord Approval Needed for Thai Twist, 337 E Rand Rd, Arlington Heights, IL 60004 [1a01d2fe3676fa46]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -973,7 +974,8 @@
           <t>Thank you, Charles! I really appreciate it. Please let me know once you&amp;#39;ve had a chance to check everything. Best Regards, Pat. On Tue, Aug 11, 2026 at 9:08 PM charles zhao &amp;lt;topchannelletters@
 buddy we can do it for you for 4000 both the store front sign and pylon sign . for the page 6, no worry. That is just the standard form we use. to confirm with you , we will build it with white return
 i think either white return with white trim cap will work fine . or black return with black trim cap will be good as well. it will give like an outline for the sign. for the raceway #8 is ok. our white
-Hi Charles, Thank you for the update. I noticed that the Zelle transfer option is not available on my account yet. I&amp;#39;m currently setting it up with the bank, which may take 1–2 business days. I</t>
+Hi Charles, Thank you for the update. I noticed that the Zelle transfer option is not available on my account yet. I&amp;#39;m currently setting it up with the bank, which may take 1–2 business days. I
+Hi Charles, The money didn&amp;#39;t go through. I&amp;#39;ll try again tomorrow. I&amp;#39;ll update you again. If it still doesn&amp;#39;t go through, I may need to make a wire transfer. Thank you Best Regards, Pat</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1273,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1296,17 +1298,19 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 14:16:26 -0500</t>
+          <t>Wed, 19 Aug 2026 10:32:37 -0500</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Thu, 30 Jul 2026 14:16:26 -0500: Re: RFQ - "FASTSIGNS" sign [19fb47514449ee89]</t>
+          <t>Thu, 30 Jul 2026 14:16:26 -0500: Re: RFQ - "FASTSIGNS" sign [19fb47514449ee89]
+Wed, 19 Aug 2026 10:32:37 -0500: Re: RFQ - "FASTSIGNS" sign [1a01aa75357c15fd]</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Hi Charles Here is the jpg file that you will be able to open. Ravi. On Thu, Jul 30, 2026 at 1:46 PM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi, I am processing the estimate right now,</t>
+          <t>Hi Charles Here is the jpg file that you will be able to open. Ravi. On Thu, Jul 30, 2026 at 1:46 PM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi, I am processing the estimate right now,
+i would say $120 for delivery Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1416,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1437,17 +1441,19 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Mon, 10 Aug 2026 08:48:15 -0400</t>
+          <t>Thu, 20 Aug 2026 15:37:21 -0500 (CDT)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Mon, 10 Aug 2026 08:48:15 -0400: Re: Card Vault face lit trimless channel letters-Indy [19febb7992a6ef2a]</t>
+          <t>Mon, 10 Aug 2026 08:48:15 -0400: Re: Card Vault face lit trimless channel letters-Indy [19febb7992a6ef2a]
+Thu, 20 Aug 2026 15:37:21 -0500 (CDT): Re: Card Vault face lit trimless channel letters-Indy [1a020e483781d90e]</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>will do . In Orlando. Will be back tomorrow Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130</t>
+          <t>will do . In Orlando. Will be back tomorrow Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130
+Just confirmed that is correct. -----Original Message----- From: &amp;quot;charles zhao&amp;quot; &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Thursday, August 20, 2026 3:09pm To: mike@signarama-bloomingdale.com</t>
         </is>
       </c>
     </row>
@@ -9773,12 +9779,13 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Thu, 23 Jul 2026 12:20:08 +0000 (UTC)</t>
+          <t>Thu, 20 Aug 2026 12:17:57 +0000 (UTC)</t>
         </is>
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>Thu, 23 Jul 2026 12:20:08 +0000 (UTC): Heng XU recommended you to their network! [19f8eeb3dc2f8790]</t>
+          <t>Thu, 23 Jul 2026 12:20:08 +0000 (UTC): Heng XU recommended you to their network! [19f8eeb3dc2f8790]
+Thu, 20 Aug 2026 12:17:57 +0000 (UTC): Heng XU recommended you to their network! [1a01f1b4f4fbbebe]</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">
@@ -9936,7 +9943,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Payment Awaiting</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -9961,7 +9968,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 15:59:01 -0500</t>
+          <t>Wed, 19 Aug 2026 14:42:46 +0000</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -9974,7 +9981,8 @@
 Tue, 18 Aug 2026 16:29:20 -0500: Life Space Digital Invoice &amp; COI from Top Channel Letters [1a016c764718db5d]
 Tue, 18 Aug 2026 16:13:42 -0500: Fwd: coi [1a016b94677bc643]
 Tue, 18 Aug 2026 15:59:01 -0500: Fwd: coi [1a016abd350fc6d3]
-Wed, 19 Aug 2026 14:42:46 +0000: Fw: Life Space Digital Invoice &amp; COI from Top Channel Letters [1a01a7998855bb61]</t>
+Wed, 19 Aug 2026 14:42:46 +0000: Fw: Life Space Digital Invoice &amp; COI from Top Channel Letters [1a01a7998855bb61]
+Thu, 20 Aug 2026 18:47:08 +0000: RE: Contractor Registration- Top Channel Letter [1a0207faa41b4bd1]</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -9986,7 +9994,8 @@
 Dear Sunny, Please see attached invoice and COI. Feel free to contact us if you have any questions. Thank you! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:
 ---------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 4:10 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan
 ---------- Forwarded message --------- From: Alex Wan &amp;lt;Alex@karstensfinancial.com&amp;gt; Date: Tue, Aug 18, 2026 at 3:53 PM Subject: coi To: Top Channel Letters Inc &amp;lt;qaprints@gmail.com&amp;gt; Alex Wan
-Hi Charles and Candy, Well received the proposal and the COI, we will confirm with you once we received approval from the building. Sunny Chen Head of Operations M: 347.993.9116 lifespacedigital.com</t>
+Hi Charles and Candy, Well received the proposal and the COI, we will confirm with you once we received approval from the building. Sunny Chen Head of Operations M: 347.993.9116 lifespacedigital.com
+Thank you for contacting the Village of Bridgeview. Your requested PIN is: 17aded4f6046 Please let me know if you have any questions or need anything else. Sincerely, Stephanie Johnson Village of</t>
         </is>
       </c>
     </row>
@@ -9998,7 +10007,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Permit</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -10023,7 +10032,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 15:16:17 -0500</t>
+          <t>Wed, 19 Aug 2026 13:12:30 -0400</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
@@ -10034,7 +10043,8 @@
 Tue, 18 Aug 2026 16:36:45 -0400: Bond Quote for Top Channel Letters Inc [1a016973e6aeb99e]
 Tue, 18 Aug 2026 15:16:17 -0500: Request a Bond of Bridgeview [1a01684757b82c05]
 Wed, 19 Aug 2026 12:27:27 -0500: Re: Quote #784591 – Unable to Upload Sign Agreement [1a01b1074dc49453]
-Wed, 19 Aug 2026 13:12:30 -0400: Bond Quote for Top Channel Letters Inc [1a01b02a6e71aed9]</t>
+Wed, 19 Aug 2026 13:12:30 -0400: Bond Quote for Top Channel Letters Inc [1a01b02a6e71aed9]
+Thu, 20 Aug 2026 12:58:50 -0400: Surety Bond Issued for Top Channel Letters Inc [1a0201c7c3aeef13]</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
@@ -10042,7 +10052,8 @@
           <t>Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609 www
 Thank you for the quote request with BondExchange, the surety partner of Karstens Financial LLC. You are approved for the following bond quote: $10000 IL License/Permit bond Bond Term Cost Due Now
 Hi, Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609
-Hello Charles, Yes, you can send the signed agreement to us and we can upload and process everythingon ourselves. Thanks, On Wed, Aug 19, 2026 at 12:10 PM charles zhao &amp;lt;topchannelletters@gmail.com</t>
+Hello Charles, Yes, you can send the signed agreement to us and we can upload and process everythingon ourselves. Thanks, On Wed, Aug 19, 2026 at 12:10 PM charles zhao &amp;lt;topchannelletters@gmail.com
+Bond Has Been issued Bond #: AM0004295 Issued Thank you for purchasing your bond with BondExchange, the surety partner of Karstens Financial LLC. Your bond number is AM0004295 . BOND FILING</t>
         </is>
       </c>
     </row>
@@ -11951,7 +11962,7 @@
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 10:07:05 -0500</t>
+          <t>Thu, 20 Aug 2026 16:33:01 -0500</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
@@ -11959,7 +11970,8 @@
           <t>Tue, 21 Jul 2026 14:25:16 -0500: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [19f8623b9f970dab]
 Fri, 14 Aug 2026 16:19:24 -0500: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a00224d432e9243]
 Mon, 17 Aug 2026 21:22:12 +0000: RE: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a0119a9d601f480]
-Tue, 18 Aug 2026 10:07:05 -0500: Re: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a015695e8912f87]</t>
+Tue, 18 Aug 2026 10:07:05 -0500: Re: EXTERNAL: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a015695e8912f87]
+Thu, 20 Aug 2026 16:33:01 -0500: Re: EXTERNAL: Sign Permit Application for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 [1a02117676396373]</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
@@ -11967,7 +11979,8 @@
           <t>Hi, Martin We are Top Channel Letters, the sign contractor for New Lenox Car Wash, 451 N VINE ST, NEW LENOX, IL 60451 We would like to apply for a sign permit for this business. The attachments include
 Hi, Lisa This is the revision for sign 3, we have updated a smaller sign to fit the requirement. Please check. Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top
 Good Afternoon, Please refer to the attached letter that our Chief Building Inspector, Ray Graefen sent regarding the review your signs. We are still in need of a response letter with electrical
-got it, thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St</t>
+got it, thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St
+Please find electrical connection for the new sign letter in attachment. Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail</t>
         </is>
       </c>
     </row>
@@ -13378,19 +13391,21 @@
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 11:39:30 -0500</t>
+          <t>Thu, 20 Aug 2026 14:09:15 -0500</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
         <is>
           <t>Wed, 12 Aug 2026 16:13:18 -0500: Re: Back lit sign - family dental [19ff7d2887ab044f]
-Fri, 14 Aug 2026 11:39:30 -0500: Re: Back lit sign - family dental [1a001249b5c5fd2e]</t>
+Fri, 14 Aug 2026 11:39:30 -0500: Re: Back lit sign - family dental [1a001249b5c5fd2e]
+Thu, 20 Aug 2026 14:09:15 -0500: Re: Back lit sign - family dental [1a02093d93ff0085]</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
         <is>
           <t>Hi, How are you doing? It has been a while since we sent the quote. What do you think of it? Please let me know if there&amp;#39;s anything you&amp;#39;d like to negociate. Hope you are having a good week.
-Thank you for letting us know! Wish you a good day sir. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile:</t>
+Thank you for letting us know! Wish you a good day sir. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile:
+I hope you are recovering well tho, I was having such a busy day last time that I didn&amp;#39;t see the part about stitches..... I am very sorry to hear that. Best Regards, Charles Zhao Top Channel</t>
         </is>
       </c>
     </row>
@@ -14546,7 +14561,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -14646,7 +14661,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Permit</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -14671,7 +14686,7 @@
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 17:17:47 +0000</t>
+          <t>Wed, 19 Aug 2026 15:07:13 +0000</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
@@ -14699,7 +14714,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Payment Awaiting</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -14724,19 +14739,21 @@
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>Mon, 17 Aug 2026 13:45:22 +0000</t>
+          <t>Thu, 20 Aug 2026 15:21:37 +0000</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
           <t>Fri, 14 Aug 2026 17:21:06 +0000: Re: Enlarging existing channel letters [1a0014ac72caa072]
-Mon, 17 Aug 2026 13:45:22 +0000: Re: Enlarging existing channel letters [1a00ff86385fac0b]</t>
+Mon, 17 Aug 2026 13:45:22 +0000: Re: Enlarging existing channel letters [1a00ff86385fac0b]
+Thu, 20 Aug 2026 15:21:37 +0000: Re: Enlarging existing channel letters [1a01fc38940c3aa2]</t>
         </is>
       </c>
       <c r="M302" t="inlineStr">
         <is>
           <t>Charles. We would like to proceed. Get Outlook for iOS From: charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Thursday, 13 August 2026 16:56:10 To: Signarama Carptenersville IL &amp;lt;
-Good morning, Charles See below and yes, I will prepare a check and send you a picture today. Also, around Noon-2oclock I will go by Zeigler&amp;#39;s and facetime you. See info below for Angry genes</t>
+Good morning, Charles See below and yes, I will prepare a check and send you a picture today. Also, around Noon-2oclock I will go by Zeigler&amp;#39;s and facetime you. See info below for Angry genes
+HI, Charles, Yes, please move forward. I forgot to send you a picture of a check for Angry Genes, sorry been very busy. I will send a picture tonight. No, I&amp;#39;m not in Joliet today. In</t>
         </is>
       </c>
     </row>
@@ -16144,12 +16161,13 @@
       </c>
       <c r="K332" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 11:54:40 -0500</t>
+          <t>Thu, 20 Aug 2026 13:36:03 -0500</t>
         </is>
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 11:54:40 -0500: Landlord Approval Needed for Red Crab， 4901 WASHINGTON AVE, RACINE, WI 53406 [1a015cbe16906dc9]</t>
+          <t>Tue, 18 Aug 2026 11:54:40 -0500: Landlord Approval Needed for Red Crab， 4901 WASHINGTON AVE, RACINE, WI 53406 [1a015cbe16906dc9]
+Thu, 20 Aug 2026 13:36:03 -0500: Landlord Approval Needed for Red Crab， 4901 WASHINGTON AVE, RACINE, WI 53406 [1a0207566f19dea7]</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
@@ -16621,12 +16639,14 @@
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 15:27:15 -0700: Pure Medical Spa Lightbox Sign Production File(J) [1a01c2305f203d3b]</t>
+          <t>Wed, 19 Aug 2026 15:27:15 -0700: Pure Medical Spa Lightbox Sign Production File(J) [1a01c2305f203d3b]
+Thu, 20 Aug 2026 13:45:12 -0500: Re: Pure Medical Spa Lightbox Sign Production File(J) [1a0207e03f550f87]</t>
         </is>
       </c>
       <c r="M342" t="inlineStr">
         <is>
-          <t>48“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St,</t>
+          <t>48“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St,
+这个面先别喷，客人可能要选用vinyl cut.做！还没定下来，但灯箱可以做了！ On Thu, Aug 20, 2026 at 1:43 PM Qa Prints &amp;lt;info.qaprints@gmail.com&amp;gt; wrote: 47“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards,</t>
         </is>
       </c>
     </row>
@@ -17138,12 +17158,18 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 16:15:15 -0500: Partnership Proposal From TopChannelLetters [1a01be0d96964497]</t>
+          <t>Wed, 19 Aug 2026 16:15:15 -0500: Partnership Proposal From TopChannelLetters [1a01be0d96964497]
+Thu, 20 Aug 2026 14:23:55 -0500: Partnership Proposal From TopChannelLetters [1a020a1498a0a02e]
+Thu, 20 Aug 2026 14:23:54 -0500: Partnership Proposal From TopChannelLetters [1a020a145df157a6]
+Thu, 20 Aug 2026 14:23:15 -0500: Partnership Proposal From TopChannelLetters [1a020a0abeb32fe2]
+Thu, 20 Aug 2026 14:23:13 -0500: Partnership Proposal From TopChannelLetters [1a020a0a581b5d18]
+Thu, 20 Aug 2026 14:23:10 -0500: Partnership Proposal From TopChannelLetters [1a020a098202dca5]</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
         <is>
-          <t>A preferred signage partnership for more consistent properties, a simpler tenant path, and program benefits tied to completed work. Top Channel Letters Chicago Fabrication Facility Partner Proposal For</t>
+          <t>A preferred signage partnership for more consistent properties, a simpler tenant path, and program benefits tied to completed work. Top Channel Letters Chicago Fabrication Facility Partner Proposal For
+Top Channel Letters Chicago Fabrication Facility Partner Proposal For your retail &amp;amp; commercial property A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
         </is>
       </c>
     </row>
@@ -17202,7 +17228,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -17484,7 +17510,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Awaiting Estimate</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -17661,6 +17687,1322 @@
       <c r="M364" t="inlineStr">
         <is>
           <t>You could get up to $10000 back in credits ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-0364</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Cricket Sign Production File (J)</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 15:45:52 -0700</t>
+        </is>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 15:45:52 -0700: Cricket Sign Production File (J) [1a0215a8319dd2c1]</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>Sign 1 完成尺寸 111.0625&amp;quot;x28.625&amp;quot; Sign 2 完成尺寸 138.8125&amp;quot;x35.8125&amp;quot; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-0365</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>SIGN-GEN-24-00486 5547 N Lovers Lane Rd Fwd: SIGN-GEN-24-00486 5547 N Lovers Lane Rd Re: SIGN-GEN-24-00486 5547 N Lovers</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>scott</t>
+        </is>
+      </c>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:31:14 +0000</t>
+        </is>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:31:14 +0000: RE: SIGN-GEN-24-00486 5547 N Lovers Lane Rd [1a020def588a9ac9]</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>Correction. The record is SIGN-GEN-26-00241 Javon Scott Plan Exam Specialist Department of Neighborhood Services Permit &amp;amp; Development Center 809 N Broadway 1st Floor, Milwaukee, WI 53202 P: (414)</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-0366</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Auto Reply from the City of Milwaukee Development Center</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>developmentcenterinf@milwaukee.gov</t>
+        </is>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:14:22 +0000</t>
+        </is>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:14:22 +0000: Auto Reply from the City of Milwaukee Development Center [1a020cf8f78e996e]</t>
+        </is>
+      </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>Thank you for contacting the City of Milwaukee Development Center. We will respond to your inquiry as soon as possible. Your opinion is important to us. Please complete our brief Permit &amp;amp;</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-0367</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Board Meeting Brief - Week of August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>admin@public.govdelivery.com</t>
+        </is>
+      </c>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:01:32 +0000</t>
+        </is>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:01:32 +0000: Board Meeting Brief - Week of August 17, 2026 [1a020c3b84fea571]</t>
+        </is>
+      </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>Having trouble viewing this email? View it as a Web page. | Bookmark and Share SUBSCRIBER SERVICES Manage Subscriptions | Unsubscribe | Help Decisions &amp;amp; Discussions from the Latest Village Meetings</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-0368</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company Re: Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>kelly_v@pentagonllc.com</t>
+        </is>
+      </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:52:11 -0500</t>
+        </is>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:52:11 -0500: Re: Partnership Proposal From A Signage Company [1a020bb2bba4bb0e]</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>Please see the attached pdf for details! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-0369</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>brian.vanevenhoven@nmrk.com</t>
+        </is>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:50:56 -0500</t>
+        </is>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:50:56 -0500: Partnership Proposal From A Signage Company [1a020ba032471aab]</t>
+        </is>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-0370</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>fred@pentagonllc.com</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:49:18 -0500</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:49:18 -0500: Partnership Proposal From A Signage Company [1a020b88502580c5]</t>
+        </is>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; 2:43 PM (5 minutes ago) to julie TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-0371</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>jwigser@dlcmgmt.com</t>
+        </is>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:49:16 -0500</t>
+        </is>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:49:16 -0500: Partnership Proposal From A Signage Company [1a020b87d43ce5aa]</t>
+        </is>
+      </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; 2:43 PM (5 minutes ago) to julie TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-0372</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>leasing@pinetree.com</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:45:33 -0500</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:45:33 -0500: Partnership Proposal From A Signage Company [1a020b517c913241]</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-0373</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>sstephens@reddevelopment.com</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:45:26 -0500</t>
+        </is>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:45:26 -0500: Partnership Proposal From A Signage Company [1a020b4fdc003234]</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-0374</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>kcaso@mccreapg.com</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:44:38 -0500</t>
+        </is>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:44:38 -0500: Partnership Proposal From A Signage Company [1a020b43efb14ae7]</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-0375</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>jtabor@regency-prop.com</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:44:09 -0500</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:44:09 -0500: Partnership Proposal From A Signage Company [1a020b3cf6ebb197]</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-0376</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>tirgens@irgens.com</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:44:02 -0500</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:44:02 -0500: Partnership Proposal From A Signage Company [1a020b3b2d4ddd29]</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-0377</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>kevin.schmoldt@ngkf.com</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:53 -0500</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:53 -0500: Partnership Proposal From A Signage Company [1a020b3932dcf555]</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-0378</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>arobbins@arcregrp.com</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:34 -0500</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:34 -0500: Partnership Proposal From A Signage Company [1a020b344a3cdf52]</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-0379</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>matt@arcregrp.com</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:25 -0500</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:25 -0500: Partnership Proposal From A Signage Company [1a020b3238ccf55a]</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-0380</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>brad@bradfordrealestate.com</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:12 -0500</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:12 -0500: Partnership Proposal From A Signage Company [1a020b2efe8b83ac]</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-0381</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>hello@centennialrec.com</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:04 -0500</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:43:04 -0500: Partnership Proposal From A Signage Company [1a020b2d3fb2da69]</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-0382</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>jwalker@centennialrec.com</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:47 -0500</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:47 -0500: Partnership Proposal From A Signage Company [1a020b28cbc1566f]</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-0383</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>bob.redican@nuveen.com</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:41 -0500</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:41 -0500: Partnership Proposal From A Signage Company [1a020b276fb40bb5]</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-0384</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>rwhis@brianproperties.com</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:32 -0500</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:32 -0500: Partnership Proposal From A Signage Company [1a020b25385dae81]</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-0385</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>mark@brianproperties.com</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:28 -0500</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:28 -0500: Partnership Proposal From A Signage Company [1a020b244838aa1c]</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-0386</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Partnership Proposal From A Signage Company</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>sb@mosaic-pd.com</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:21 -0500</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 14:42:21 -0500: Partnership Proposal From A Signage Company [1a020b22816b4eaa]</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>TOP CHANNEL LETTERS CHICAGO FABRICATION FACILITY PARTNER PROPOSAL FOR YOUR RETAIL &amp;amp; COMMERCIAL PROPERTY A Partnership Invitation for Your Tenant Signage Program Collaborate with us for a consistent</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-0387</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Completed: You're copied on "Bedford Nail Spa Sign Rendering 26-6"</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>adobesign@adobesign.com</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 09:58:35 -0700 (PDT)</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 09:58:35 -0700 (PDT): Completed: You're copied on "Bedford Nail Spa Sign Rendering 26-6" [1a0201c3cf9947e7]</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>Attached is the final agreement for your reference. QA PRINTS cc&amp;#39;d you on Bedford Nail Spa Sign Rendering 26-6 Open agreement Attached is the final agreement between: QA PRINTS John Hurley Read it</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-0388</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Card Vault Indy trimless channel letters</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>mike@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 11:32:03 -0500 (CDT)</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 11:32:03 -0500 (CDT): Card Vault Indy trimless channel letters [1a02003f4d7dff80]</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>Can you price out these channel letters? Two sets! Shipped to INDY</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-0389</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>yooyee logo</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>yuyi.zhouchicago@gmail.com</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 18:07:45 -0500</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 18:07:45 -0500: yooyee logo [1a01c48133f31e97]</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>Hi here is our logo. let me know if you need anything else Thank you</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-0390</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Interior illuminated sign</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>signarama woodridge</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:47:01 +0000</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 17:47:01 +0000: Re: Interior illuminated sign [1a01b223c0d3440b]</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>It should be this size and a raceway would need to be produced as well. Thanks! From: charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Tuesday, August 18, 2026 4:04 PM To: Signarama Woodridge, IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-0391</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Presotea - Sign Info</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>tony.liu@presoteacorporation.com</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 10:44:33 -0500</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Wed, 19 Aug 2026 10:44:33 -0500: Re: Presotea - Sign Info [1a01ab20de8d3f82]</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>Can You give me a call when you have time? my number is 3124042130. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily order sync: 2026-08-21
</commit_message>
<xml_diff>
--- a/data/orders.xlsx
+++ b/data/orders.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M392"/>
+  <dimension ref="A1:M406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1202,19 +1202,21 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Sun, 16 Aug 2026 22:42:26 -0500</t>
+          <t>Fri, 21 Aug 2026 13:58:58 -0500</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>Wed, 5 Aug 2026 14:20:15 -0400: Re: TopChannelLetters - Referred by Jovim from inoprints [19fd327c4360bcd0]
-Sun, 16 Aug 2026 22:42:26 -0500: Re: TopChannelLetters - Referred by Jovim from inoprints [1a00dd03bb458bb8]</t>
+Sun, 16 Aug 2026 22:42:26 -0500: Re: TopChannelLetters - Referred by Jovim from inoprints [1a00dd03bb458bb8]
+Fri, 21 Aug 2026 13:58:58 -0500: Re: TopChannelLetters - Referred by Jovim from inoprints [1a025b0f905834af]</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>Can I send someone to measure the building size ? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404
-HI, Yosf, Please check the sample of the backlit channel letters we made for other businesses. Do you like the silver color or the gold color? and do you think you can stop by our sign shop and talk</t>
+HI, Yosf, Please check the sample of the backlit channel letters we made for other businesses. Do you like the silver color or the gold color? and do you think you can stop by our sign shop and talk
+You think it would look better than white? It looks white in the mockup On Fri, Aug 21, 2026 at 11:32 AM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: yup. it is back lit channel letters.</t>
         </is>
       </c>
     </row>
@@ -1298,19 +1300,21 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 10:32:37 -0500</t>
+          <t>Thu, 20 Aug 2026 13:34:55 -0500</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>Thu, 30 Jul 2026 14:16:26 -0500: Re: RFQ - "FASTSIGNS" sign [19fb47514449ee89]
-Wed, 19 Aug 2026 10:32:37 -0500: Re: RFQ - "FASTSIGNS" sign [1a01aa75357c15fd]</t>
+Wed, 19 Aug 2026 10:32:37 -0500: Re: RFQ - "FASTSIGNS" sign [1a01aa75357c15fd]
+Thu, 20 Aug 2026 13:34:55 -0500: Re: RFQ - "FASTSIGNS" sign [1a020749655ba9e8]</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>Hi Charles Here is the jpg file that you will be able to open. Ravi. On Thu, Jul 30, 2026 at 1:46 PM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Hi, I am processing the estimate right now,
-i would say $120 for delivery Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St</t>
+i would say $120 for delivery Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St
+Yes. Next Tuesday. On Monday I will be on my return flight and wont reach back until late afternoon. I will try to remember to remind you. Thanks Ravi. On Thu, Aug 20, 2026 at 1:32 PM charles zhao &amp;lt;</t>
         </is>
       </c>
     </row>
@@ -2432,17 +2436,19 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Fri, 07 Aug 2026 02:39:44 +0000 (UTC)</t>
+          <t>Fri, 21 Aug 2026 22:18:35 +0000 (UTC)</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Fri, 07 Aug 2026 02:39:44 +0000 (UTC): Invoice - Reminder: Your payment to Top Channel Letters is due [19fda1740f9d4c48]</t>
+          <t>Fri, 07 Aug 2026 02:39:44 +0000 (UTC): Invoice - Reminder: Your payment to Top Channel Letters is due [19fda1740f9d4c48]
+Fri, 21 Aug 2026 22:18:35 +0000 (UTC): Invoice - Reminder: Your payment to Top Channel Letters is due [1a02667901c19f39]</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Your invoice is ready! BALANCE DUE$4400.00 Total $8800.00 View and pay Terms &amp;amp; Conditions ***A 4% processing fee will be applied to all credit card payments*** 1. All Sold Goods are not returnable</t>
+          <t>Your invoice is ready! BALANCE DUE$4400.00 Total $8800.00 View and pay Terms &amp;amp; Conditions ***A 4% processing fee will be applied to all credit card payments*** 1. All Sold Goods are not returnable
+Your invoice is ready! BALANCE DUE$1300.00 View and pay Terms &amp;amp; Conditions ***A 4% processing fee will be applied to all credit card payments*** 1. All Sold Goods are not returnable and refundable.</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9949,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Payment Awaiting</t>
+          <t>Permit</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -9968,7 +9974,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 14:42:46 +0000</t>
+          <t>Thu, 20 Aug 2026 18:47:08 +0000</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -10007,7 +10013,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Permit</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -10032,7 +10038,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 13:12:30 -0400</t>
+          <t>Thu, 20 Aug 2026 12:58:50 -0400</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
@@ -10044,7 +10050,8 @@
 Tue, 18 Aug 2026 15:16:17 -0500: Request a Bond of Bridgeview [1a01684757b82c05]
 Wed, 19 Aug 2026 12:27:27 -0500: Re: Quote #784591 – Unable to Upload Sign Agreement [1a01b1074dc49453]
 Wed, 19 Aug 2026 13:12:30 -0400: Bond Quote for Top Channel Letters Inc [1a01b02a6e71aed9]
-Thu, 20 Aug 2026 12:58:50 -0400: Surety Bond Issued for Top Channel Letters Inc [1a0201c7c3aeef13]</t>
+Thu, 20 Aug 2026 12:58:50 -0400: Surety Bond Issued for Top Channel Letters Inc [1a0201c7c3aeef13]
+Thu, 20 Aug 2026 12:23:05 -0500: Re: Quote #784591 – Unable to Upload Sign Agreement [1a02032f6ffcfca5]</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
@@ -10053,7 +10060,8 @@
 Thank you for the quote request with BondExchange, the surety partner of Karstens Financial LLC. You are approved for the following bond quote: $10000 IL License/Permit bond Bond Term Cost Due Now
 Hi, Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago, IL 60609
 Hello Charles, Yes, you can send the signed agreement to us and we can upload and process everythingon ourselves. Thanks, On Wed, Aug 19, 2026 at 12:10 PM charles zhao &amp;lt;topchannelletters@gmail.com
-Bond Has Been issued Bond #: AM0004295 Issued Thank you for purchasing your bond with BondExchange, the surety partner of Karstens Financial LLC. Your bond number is AM0004295 . BOND FILING</t>
+Bond Has Been issued Bond #: AM0004295 Issued Thank you for purchasing your bond with BondExchange, the surety partner of Karstens Financial LLC. Your bond number is AM0004295 . BOND FILING
+Hello Charles, You are welcome, anytime! Thanks, On Thu, Aug 20, 2026 at 12:08 PM charles zhao &amp;lt;topchannelletters@gmail.com&amp;gt; wrote: Thank you for your help. Best Regards, Charles Zhao Top Channel</t>
         </is>
       </c>
     </row>
@@ -12158,12 +12166,13 @@
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Tue, 21 Jul 2026 11:17:10 -0700 (PDT)</t>
+          <t>Fri, 21 Aug 2026 12:22:01 -0700 (PDT)</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>Tue, 21 Jul 2026 11:17:10 -0700 (PDT): Your AT&amp;T online bill is ready to be viewed [19f85e5697c63006]</t>
+          <t>Tue, 21 Jul 2026 11:17:10 -0700 (PDT): Your AT&amp;T online bill is ready to be viewed [19f85e5697c63006]
+Fri, 21 Aug 2026 12:22:01 -0700 (PDT): Your AT&amp;T online bill is ready to be viewed [1a025c5ea033b861]</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
@@ -13151,7 +13160,7 @@
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Fri, 14 Aug 2026 12:46:31 -0400 (EDT)</t>
+          <t>Fri, 21 Aug 2026 16:43:51 -0400 (EDT)</t>
         </is>
       </c>
       <c r="L269" t="inlineStr">
@@ -13159,12 +13168,14 @@
           <t>Wed, 12 Aug 2026 18:12:18 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ff8088e344e873]
 Thu, 13 Aug 2026 15:12:21 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [19ffc8a2a1707ef0]
 Fri, 14 Aug 2026 12:46:31 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a0012b032f8c76d]
-Sat, 15 Aug 2026 10:57:47 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a005edd40ae423a]</t>
+Sat, 15 Aug 2026 10:57:47 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a005edd40ae423a]
+Fri, 21 Aug 2026 16:43:51 -0400 (EDT): Register Today for the Inaugural Great Lakes Sign Association Conference and Sign Expo--September 9-10, 2026 [1a02610d290e2495]</t>
         </is>
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t>Logo contest and sign design entries due by 08/28/2026! Minnesota Sign Association (MSA) REGISTRATION OPEN! ﻿ GLSA FALL CONFERENCE Register to join your industry peers for the inaugural conference of</t>
+          <t>Logo contest and sign design entries due by 08/28/2026! Minnesota Sign Association (MSA) REGISTRATION OPEN! ﻿ GLSA FALL CONFERENCE Register to join your industry peers for the inaugural conference of
+Logo contest and sign design entries due by 08/28/2026! Minnesota Sign Association (MSA) Logo design and sign design submissions due date is 1 week from today. Don&amp;#39;t forget to submit and register</t>
         </is>
       </c>
     </row>
@@ -14561,7 +14572,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Installation</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -14586,7 +14597,7 @@
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 18:22:51 +0000</t>
+          <t>Fri, 21 Aug 2026 15:42:45 +0000</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
@@ -14594,7 +14605,8 @@
           <t>Fri, 14 Aug 2026 17:01:14 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0024b5160293ad]
 Sun, 16 Aug 2026 23:02:52 -0500: Re: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a00de2eea056286]
 Tue, 18 Aug 2026 22:42:40 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a0170b0c263cade]
-Wed, 19 Aug 2026 18:22:51 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a01b4377a1ae38c]</t>
+Wed, 19 Aug 2026 18:22:51 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a01b4377a1ae38c]
+Fri, 21 Aug 2026 15:42:45 +0000: RE: Request for Proposal – Stretch Zone Signage | 1733 W. Kirby Ave., Champaign [1a024fdd3260352f]</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
@@ -14602,7 +14614,8 @@
           <t>Hello Charles, I am in the process of opening a new Stretch Zone studio at 1733 W. Kirby Avenue in Champaign and would like to request a proposal for the fabrication and installation of our exterior
 Hi, is this sport clip your shop? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W
 Hi Lowa, I have requested of Landlord&amp;#39;s broker any exterior elevations they may have for reference. Your signage is a great investment for your business. This pursuit is the tenant&amp;#39;s own with
-Hi Lowa, Landlord nor its broker have any elevation drawings for reference nor prior signage exhibits on this space in Old Farm. Your signage renderings will all have to be drawn up from the pictures/</t>
+Hi Lowa, Landlord nor its broker have any elevation drawings for reference nor prior signage exhibits on this space in Old Farm. Your signage renderings will all have to be drawn up from the pictures/
+Good morning, As the signage progresses along, hopefully the lease will be sent out early next week, and the renderings will need to be submitted to the Landlord for review and approval, including the</t>
         </is>
       </c>
     </row>
@@ -16587,17 +16600,19 @@
       </c>
       <c r="K341" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 17:29:21 -0500</t>
+          <t>Fri, 21 Aug 2026 16:09:52 -0500</t>
         </is>
       </c>
       <c r="L341" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 17:29:21 -0500: Landloard Approval Needed for Ou's Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 [1a01c24a35502c2b]</t>
+          <t>Wed, 19 Aug 2026 17:29:21 -0500: Landloard Approval Needed for Ou's Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 [1a01c24a35502c2b]
+Fri, 21 Aug 2026 16:09:52 -0500: Re: Landloard Approval Needed for Ou's Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 [1a026288ff58fa7f]</t>
         </is>
       </c>
       <c r="M341" t="inlineStr">
         <is>
-          <t>Dear Landlord, This is Top Channel Letters, we are the sign contractor for your tenant Ou&amp;#39;s Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 Please see attached, you will find the</t>
+          <t>Dear Landlord, This is Top Channel Letters, we are the sign contractor for your tenant Ou&amp;#39;s Hibachi Pylon Sign, 2557 Capital Ave SW, Battle Creek, MI 49015 Please see attached, you will find the
+Hi, Dear landlord A reminder for my previous email. Please find the sign plan in the attachment Thank you so much! Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email:</t>
         </is>
       </c>
     </row>
@@ -16634,19 +16649,21 @@
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 15:27:15 -0700</t>
+          <t>Thu, 20 Aug 2026 10:36:03 -0700</t>
         </is>
       </c>
       <c r="L342" t="inlineStr">
         <is>
           <t>Wed, 19 Aug 2026 15:27:15 -0700: Pure Medical Spa Lightbox Sign Production File(J) [1a01c2305f203d3b]
-Thu, 20 Aug 2026 13:45:12 -0500: Re: Pure Medical Spa Lightbox Sign Production File(J) [1a0207e03f550f87]</t>
+Thu, 20 Aug 2026 13:45:12 -0500: Re: Pure Medical Spa Lightbox Sign Production File(J) [1a0207e03f550f87]
+Thu, 20 Aug 2026 10:36:03 -0700: Re: Pure Medical Spa Lightbox Sign Production File(J) [1a0203ec91075373]</t>
         </is>
       </c>
       <c r="M342" t="inlineStr">
         <is>
           <t>48“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St,
-这个面先别喷，客人可能要选用vinyl cut.做！还没定下来，但灯箱可以做了！ On Thu, Aug 20, 2026 at 1:43 PM Qa Prints &amp;lt;info.qaprints@gmail.com&amp;gt; wrote: 47“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards,</t>
+这个面先别喷，客人可能要选用vinyl cut.做！还没定下来，但灯箱可以做了！ On Thu, Aug 20, 2026 at 1:43 PM Qa Prints &amp;lt;info.qaprints@gmail.com&amp;gt; wrote: 47“ 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards,
+47&amp;#39;&amp;#39;文件。 灯箱，单面。 6&amp;#39; plug 3/5&amp;quot; black return, black trim cap 3/4 Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420</t>
         </is>
       </c>
     </row>
@@ -17153,7 +17170,7 @@
       </c>
       <c r="K353" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 16:15:15 -0500</t>
+          <t>Thu, 20 Aug 2026 14:23:10 -0500</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
@@ -17253,17 +17270,19 @@
       </c>
       <c r="K355" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 14:24:27 -0500</t>
+          <t>Thu, 20 Aug 2026 17:45:56 -0500 (CDT)</t>
         </is>
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 14:24:27 -0500: Re: Halo lit acrylic back channel letter with chrome finish [1a01b7b6c7543d45]</t>
+          <t>Wed, 19 Aug 2026 14:24:27 -0500: Re: Halo lit acrylic back channel letter with chrome finish [1a01b7b6c7543d45]
+Thu, 20 Aug 2026 17:45:56 -0500 (CDT): Re: Halo lit acrylic back channel letter with chrome finish [1a0215a3ce57fb3e]</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
         <is>
-          <t>Hi, Thank you for contacting us, we are working on it now, will get back to you soon. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com</t>
+          <t>Hi, Thank you for contacting us, we are working on it now, will get back to you soon. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com
+ok thank you I sent everything to the customer -----Original Message----- From: &amp;quot;charles zhao&amp;quot; &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Thursday, August 20, 2026 4:23pm To: mike@signarama-</t>
         </is>
       </c>
     </row>
@@ -17535,17 +17554,19 @@
       </c>
       <c r="K361" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 11:17:54 -0500</t>
+          <t>Thu, 20 Aug 2026 17:04:24 -0500 (CDT)</t>
         </is>
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>Wed, 19 Aug 2026 11:17:54 -0500: Re: FW: Savvy Sliders [1a01ad09c47b51a7]</t>
+          <t>Wed, 19 Aug 2026 11:17:54 -0500: Re: FW: Savvy Sliders [1a01ad09c47b51a7]
+Thu, 20 Aug 2026 17:04:24 -0500 (CDT): Re: FW: Savvy Sliders [1a0213407f1ef033]</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
         <is>
-          <t>give me a call bro Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL,</t>
+          <t>give me a call bro Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL,
+Thank you i will keep you posted. -----Original Message----- From: &amp;quot;charles zhao&amp;quot; &amp;lt;topchannelletters@gmail.com&amp;gt; Sent: Thursday, August 20, 2026 4:43pm To: aaron@signarama-bloomingdale.</t>
         </is>
       </c>
     </row>
@@ -19003,6 +19024,664 @@
       <c r="M392" t="inlineStr">
         <is>
           <t>Can You give me a call when you have time? my number is 3124042130. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-0392</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Prosper - Channel Letters Re: FW: Prosper - Channel Letters Re: FW: Prosper - Channel Letters</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>aaron@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 17:34:26 -0500 (CDT)</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 17:34:26 -0500 (CDT): Re: FW: Prosper - Channel Letters [1a026760eb283e74]</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>you can make any raceway you want to the letters below can be individual channel letters. If you want -----Original Message----- From: &amp;quot;charles zhao&amp;quot; &amp;lt;topchannelletters@gmail.com&amp;gt; Sent:</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-0393</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>FBS PROJECT 38-2026 HomeSmart Sign Production File (J)</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Vinyl Graphics</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 15:33:08 -0700</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 15:33:08 -0700: FBS PROJECT 38-2026 HomeSmart Sign Production File (J) [1a026753d62bcd43]</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>168&amp;quot;x31.53&amp;quot; 一套 - Raceway color sw 7071 gray screen - Black Return, Black trimcap. - Logo和Home signface相同颜色。 - Need ul sticker and a disconnect switch on it. Best Regards, Charles Zhao</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-0394</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Uptown Cheapskate estimate needed</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>aaron@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 17:32:12 -0500 (CDT)</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 17:32:12 -0500 (CDT): Uptown Cheapskate estimate needed [1a0267404b149cb4]</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>Charles another one i need quoted. Thank you, Aaron</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-0395</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>FBS PROJECT 37-2026 Rosati's Pizza Sign Production File (J)</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Vinyl Graphics</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 14:43:18 -0700</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 14:43:18 -0700: FBS PROJECT 37-2026 Rosati's Pizza Sign Production File (J) [1a026479567b445a]</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>21.36&amp;quot; x 245&amp;quot; 两套 Black Trimcap, Black Return Ul sticker on all and also a power supply box to put the power suppy in. Best Regards, Charles Zhao QaPrints Best Price for large quantity prints</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-0396</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Only) Lava Crab Sign</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 13:54:30 -0700</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 13:54:30 -0700: (Estimate Only) Lava Crab Sign [1a0261ace20de618]</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>1. 入口招牌 logo灯箱 56&amp;#39;&amp;#39; 发光字 92.25&amp;#39;&amp;#39;x20.5&amp;#39;&amp;#39; tagline 89&amp;#39;&amp;#39;x6.5&amp;#39;&amp;#39; 2. 侧面主街招牌 logo灯箱 44&amp;quot; 发光字 字高约37.8&amp;#39;&amp;#39; tagline 235&amp;quot;x15.9&amp;quot; 3. 街边招牌 *客人提供的高度和宽度对不上，需确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-0397</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>(Quotation Need)  Wiring Diagram For New Lenox Car Wash Re: (Quotation Need) Wiring Diagram For New Lenox Car Wash Re: (</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>adnandavid27@yahoo.com</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 15:22:26 -0500</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 15:22:26 -0500: Re: (Quotation Need) Wiring Diagram For New Lenox Car Wash [1a025fd6354818a6]</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>Let me call u Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-0398</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>RE: St Sophia Re: FW: RE: St Sophia Re: St Sophia</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>aaron@signarama-bloomingdale.com</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 12:45:38 -0500</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 12:45:38 -0500: Re: St Sophia [1a0256dd06d69a3f]</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>Let me check Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-6606 | Mobile: 312-404-2130 1111 W 35th St 6th FL, Chicago,</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-0399</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Awaiting Estimate</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Only) Dragon Kitchen (Fulton) Sign</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>info.qaprints@gmail.com</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 10:15:32 -0700</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 10:15:32 -0700: (Estimate Only) Dragon Kitchen (Fulton) Sign [1a02552566d326c7]</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>355&amp;#39;&amp;#39;x31&amp;#39;&amp;#39; Best Regards, Charles Zhao QaPrints Best Price for large quantity prints P: (312) 239-6606 E: info.qaprints@gmail.com 3420 S Morgan St, Chicago, IL 60608 www.qaprints.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-0400</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Payment received: Invoice #182862-(Magic Sign Design)</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>quickbooks@notification.intuit.com</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 16:42:58 +0000 (UTC)</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 16:42:58 +0000 (UTC): Payment received: Invoice #182862-(Magic Sign Design) [1a025344ba0e03e6]</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>Intuit QuickBooks View sale $1700.00 Payment has been received Payment details Paid to Top Channel Letters Customer name Magic Sign Design Customer email magicsigndesign@gmail.com Invoice no. 182862</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-0401</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>PROJECT 38-2026 ( HOMESMART NAPERVILLE) Re: PROJECT 38-2026 ( HOMESMART NAPERVILLE)</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>getyoursigns@gmail.com</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 11:24:37 -0500</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 11:24:37 -0500: Re: PROJECT 38-2026 ( HOMESMART NAPERVILLE) [1a025237a08a7e08]</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>how do you want the logo to put together , with a backer plate or what? Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-0402</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>PROJECT 37-2026 ( ROSATI'S CARMEL) qty 2 Re: PROJECT 37-2026 ( ROSATI'S CARMEL) qty 2</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>getyoursigns@gmail.com</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 10:44:47 -0500</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 10:44:47 -0500: Re: PROJECT 37-2026 ( ROSATI'S CARMEL) qty 2 [1a024ff02c8c7f0a]</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>Hi Shannon, Order received, we will keep it going! Nice to collaborate. Best Regards, Charles Zhao Top Channel Letters Top Quality Signs at Top Speed! Email: topchannelletters@gmail.com Phone: 312-239-</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-0403</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>451 Vine Signs</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>rgraefen@newlenox.net</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 15:17:39 +0000</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 15:17:39 +0000: 451 Vine Signs [1a024e696b8e0981]</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>We have completed our second review for the sign permits. Please see the attached letter. Ray Graefen Chief Building Inspector (815) 462-6492 (office) (815) 462-6469 (fax) Village of New Lenox 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-0404</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>SIGN-GEN-24-00486 5547 N Lovers Lane Rd Re: SIGN-GEN-24-00486 5547 N Lovers Lane Rd Fwd: SIGN-GEN-24-00486 5547 N Lovers</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Channel Letters</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>scott</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:31:14 +0000</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Thu, 20 Aug 2026 20:31:14 +0000: RE: SIGN-GEN-24-00486 5547 N Lovers Lane Rd [1a020def588a9ac9]</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>Correction. The record is SIGN-GEN-26-00241 Javon Scott Plan Exam Specialist Department of Neighborhood Services Permit &amp;amp; Development Center 809 N Broadway 1st Floor, Milwaukee, WI 53202 P: (414)</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-0405</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>You're meant to be a business owner. Start now.</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Unknown / Review</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>email@email.shopify.com</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 09:46:03 +0000</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Fri, 21 Aug 2026 09:46:03 +0000: You're meant to be a business owner. Start now. [1a023b6982fbe248]</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>Sign up for a plan to build your store without interruption. ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏ ﻿͏</t>
         </is>
       </c>
     </row>

</xml_diff>